<commit_message>
added entry to translation xlsx
</commit_message>
<xml_diff>
--- a/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
+++ b/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC64C83B-1430-44AD-8FCF-CB9C3972A0A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F5A3949-6F06-4366-A4CE-A0D8643C3E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="24" yWindow="120" windowWidth="23016" windowHeight="12216" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1660" uniqueCount="787">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1667" uniqueCount="791">
   <si>
     <t>interview</t>
   </si>
@@ -22755,6 +22755,19 @@
       </rPr>
       <t>% endif</t>
     </r>
+  </si>
+  <si>
+    <t>docassemble.playground3PoAHealthCareSpanish:power_of_attorney_for_health_care.yml</t>
+  </si>
+  <si>
+    <t>64ed875eeb30496e64d73b9be2b5030e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">About the witness
+</t>
+  </si>
+  <si>
+    <t>Acerca del testigo</t>
   </si>
 </sst>
 </file>
@@ -23219,7 +23232,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H237"/>
+  <dimension ref="A1:H238"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="61.109375" customWidth="1"/>
@@ -29391,6 +29404,32 @@
         <v>602</v>
       </c>
     </row>
+    <row r="238" spans="1:8">
+      <c r="A238" t="s">
+        <v>787</v>
+      </c>
+      <c r="B238" t="s">
+        <v>599</v>
+      </c>
+      <c r="C238">
+        <v>1</v>
+      </c>
+      <c r="D238" t="s">
+        <v>788</v>
+      </c>
+      <c r="E238" t="s">
+        <v>11</v>
+      </c>
+      <c r="F238" t="s">
+        <v>12</v>
+      </c>
+      <c r="G238" t="s">
+        <v>789</v>
+      </c>
+      <c r="H238" s="4" t="s">
+        <v>790</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
trying to fix download page translation
</commit_message>
<xml_diff>
--- a/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
+++ b/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F5A3949-6F06-4366-A4CE-A0D8643C3E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5533994-9589-4A66-A80F-83B63FDC31AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24" yWindow="120" windowWidth="23016" windowHeight="12216" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -16116,118 +16116,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if not user_logged_in():
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[${fa_icon("sign-in-alt", color="#0079d0", size="sm")} **Iniciar sesión**]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${url_of('login', next=interview_url())}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>) o [**crear**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${url_of('register', next=interview_url())}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">) una cuenta de Formularios Guiados de ILAO para guardar tu progreso (opcional).
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ action_button_html(interview_url(i="docassemble.ILAO:feedback.yml", easy_form_interview=ilao_easy_form_url, easy_form_title=ilao_easy_form_title, easy_form_page=current_context().question_id, easy_form_variable=current_context().variable, local=False,reset=1), label='^^comment^^ ¿Fue útil este programa?', color="#181c36", size="md", new_window=True) }</t>
-    </r>
-  </si>
-  <si>
     <t>Empodérate de tu Futuro - Pérdida de memoria</t>
   </si>
   <si>
@@ -21509,6 +21397,1074 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Tus formularios están listos. Puedes verlos y descargarlos abajo. Haz clic en **Hacer cambios** para corregir cualquier error.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if user_path == "Shirley":
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[YOUTUBE NE0faXuz5v4]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% elif user_path == "Frederico" or user_path == "Federico":
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[YOUTUBE g5Vdv0hWJ6g]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% elif user_path == "Lisa":
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[YOUTUBE F2QbdrhcZ0g]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Lee las instrucciones para saber qué hacer después.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ action_button_html(url_action('review_answers'), label=':edit: Hacer cambios', color='success', size="md") }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ al_user_bundle.download_list_html() }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+&amp;nbsp;
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ al_user_bundle.send_button_html(show_editable_checkbox=False) }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+**Nota:** El Poder Notarial debe firmarse frente a al menos un testigo para que sea válido.
+¡Gracias por usar los Formularios Guiados de ILAO!</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Bienvenido(a) al Formulario Guiado de Poder Notarial para el Cuidado de la Salud de Illinois Legal Aid Online.
+Este programa te ayuda a crear documentos que le dan a alguien en quien confías el poder legal para tomar decisiones sobre tu atención médica. Esto significa que esa persona podrá tomar decisiones sobre tu atención médica cuando no puedas hacerlo tú mismo(a). También puedes permitir que esa persona tome decisiones sobre tu atención médica antes, si así lo decides.
+Este programa incluye videos con información sobre cómo hacer un Poder Notarial para el Cuidado de la Salud. No tienes que verlos, pero pueden serte útiles.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if user_path == "Shirley":
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">[YOUTUBE 7qy101TRdiI]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% elif user_path == "Frederico" or user_path == "Federico":
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">[YOUTUBE GR9t6ygX13g]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% elif user_path == "Lisa":
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">[YOUTUBE h2ZGl568xHo]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Para obtener más información, lee el artículo de ILAO sobre los [**Conceptos Básicos del Poder Notarial para el Cuidado de la Salud**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/legal-information/setting-power-attorney-healthcare</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Después de descargar tus formularios, tendrás que firmar el documento frente a un testigo. El testigo también tendrá que firmar el documento. No necesitas saber quién será el testigo para usar este programa.
+Después de que el formulario esté firmado, querrás entregar copias del poder notarial a tu agente, así como a tus proveedores de atención médica. Tus formularios incluirán instrucciones con más información.
+Para obtener más información, lee el artículo de ILAO sobre los [**Conceptos Básicos del Poder Notarial para el Cuidado de la Salud**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/legal-information/setting-power-attorney-healthcare</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).
+Si deseas saber más sobre la planificación en caso de discapacidad o el cuidado al final de la vida, puedes revisar la guía de ILAO y CDEL [**Empodérate de tu Futuro**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ preview.url_for() }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Tu agente es una persona en quien confías y que eliges para tomar decisiones sobre tu atención médica y cuidado de tu salud por ti, si alguna vez necesitas ayuda. 
+Tu agente debe tener al menos 18 años de edad. Tu agente no tiene que ser un familiar, pero debe ser alguien en quien confíes. Tu agente no necesita ser ciudadano de los Estados Unidos. 
+Puedes seleccionar agentes sucesores como respaldo si el primer agente no puede tomar estas decisiones.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">${collapse_template(video_who_agent)}
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+ **Nota:** Si puedes comunicarte y entender tus opciones, tú eres quien toma las decisiones.
+Para obtener más información, lee el artículo de ILAO sobre [**Conceptos Básicos del Poder Notarial para el Cuidado de la Salud**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/legal-information/setting-power-attorney-healthcare</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>No. Puedes nombrar como agente a alguien que vive fuera de los Estados Unidos. El agente no necesita ser ciudadano de los Estados Unidos. Sin embargo, pueden haber problemas si un banco u otra institución financiera no puede comunicarse con esa persona. Es posible que desees consultar a un abogado para obtener asesoramiento. Usa [**Obtener ayuda legal**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/get-legal-help</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) para encontrar servicios legales gratuitos o de bajo costo en tu área.
+Para direcciones internacionales, habrá espacio para ingresar la dirección en dos líneas. Debes escribir la dirección internacional usando el alfabeto inglés.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if for_yourself == True:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Puedes cambiar de opinión y poner fin a tu Poder Notarial para el Cuidado de la Salud en cualquier momento. Esto se llama revocación.
+La revocación significa que dejas de permitir que </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${agent.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tome decisiones por ti. Para obtener más información, lee el artículo de ILAO sobre [**poner fin a un Poder Notarial**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/legal-information/ending-power-attorney-0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).
+Puedes poner fin a un Poder Notarial haciendo una revocación formal. Para hacer una Revocación de Poder Notarial, usa el [**Formulario Guiado de Revocación de Poder Notarial**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/legal-information/power-attorney-revocation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% else:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> puede cambiar de opinión y poner fin a su Poder Notarial para el Cuidado de la Salud en cualquier momento. Esto se llama revocación.
+La revocación significa que </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> deja de permitir que </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${agent.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> tome decisiones en su nombre. Para obtener más información, lee el artículo de ILAO sobre [**poner fin a un Poder Notarial**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/legal-information/ending-power-attorney-0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> puede poner fin a un Poder Notarial haciendo una revocación formal. Para hacer una Revocación de Poder Notarial, usa el [**Formulario Guiado de Revocación de Poder Notarial**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/legal-information/power-attorney-revocation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>% endif</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>No. Puedes nombrar como agente sucesor a alguien que vive fuera de los Estados Unidos. El agente sucesor no necesita ser ciudadano de los Estados Unidos. Sin embargo, puede haber problemas si un banco u otra institución financiera no puede comunicarse con esa persona. Es posible que desees consultar con un abogado. Usa [**Obtener ayuda legal**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/get-legal-help</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) para encontrar servicios legales gratuitos o de bajo costo en tu área.
+Para direcciones internacionales, habrá espacio para ingresar la dirección en dos líneas.
+Debes escribir la dirección internacional usando el alfabeto inglés.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Tus formularios están adjuntos.
+¡Gracias por usar los Formularios Guiados de ILAO!
+[Illinois Legal Aid Online](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">**Estás haciendo estos formularios para:**
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if for_yourself == True:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Para mí
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% else:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Para otra persona
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>% endif</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">**Your treatment instructions:**
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if quality_of_life == 'quality':
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The quality of my life is more important than the length of my life.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+% if quality_of_life == 'longevity':
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">I want my life to be prolonged to the greatest extent possible.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+% if quality_of_life == 'do_not':
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">I do not want to decide this now.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>**Tus instrucciones sobre tratamiento:**</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+% if quality_of_life == 'quality':
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">La calidad de mi vida es más importante que la duración de mi vida.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+% if quality_of_life == 'longevity':
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Quiero que mi vida se prolongue en la mayor medida posible.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+% if quality_of_life == 'do_not':
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">No quiero decidir esto ahora.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>% endif</t>
+    </r>
+  </si>
+  <si>
+    <t>docassemble.playground3PoAHealthCareSpanish:power_of_attorney_for_health_care.yml</t>
+  </si>
+  <si>
+    <t>64ed875eeb30496e64d73b9be2b5030e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">About the witness
+</t>
+  </si>
+  <si>
+    <t>Acerca del testigo</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">Your forms are ready. View and download your forms below. Click **Make changes** to fix any mistakes.
 </t>
     </r>
@@ -21711,37 +22667,91 @@
   <si>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Tus formularios están listos. Puedes verlos y descargarlos abajo. Haz clic en **Hacer cambios** para corregir cualquier error.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if user_path == "Shirley":
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[YOUTUBE NE0faXuz5v4]</t>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if not user_logged_in():
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[${fa_icon("sign-in-alt", color="#0079d0", size="sm")} **Iniciar sesión**]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${url_of('login', next=interview_url())}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) o [**crear**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${url_of('register', next=interview_url())}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">) una cuenta de Formularios Guiados de ILAO para guardar tu progreso (opcional).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
     </r>
     <r>
       <rPr>
@@ -21758,1016 +22768,13 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% elif user_path == "Frederico" or user_path == "Federico":
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[YOUTUBE g5Vdv0hWJ6g]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% elif user_path == "Lisa":
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[YOUTUBE F2QbdrhcZ0g]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Lee las instrucciones para saber qué hacer después.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ action_button_html(url_action('review_answers'), label=':edit: Hacer cambios', color='success', size="md") }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ al_user_bundle.download_list_html() }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-&amp;nbsp;
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ al_user_bundle.send_button_html(show_editable_checkbox=False) }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-**Nota:** El Poder Notarial debe firmarse frente a al menos un testigo para que sea válido.
-¡Gracias por usar los Formularios Guiados de ILAO!</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Bienvenido(a) al Formulario Guiado de Poder Notarial para el Cuidado de la Salud de Illinois Legal Aid Online.
-Este programa te ayuda a crear documentos que le dan a alguien en quien confías el poder legal para tomar decisiones sobre tu atención médica. Esto significa que esa persona podrá tomar decisiones sobre tu atención médica cuando no puedas hacerlo tú mismo(a). También puedes permitir que esa persona tome decisiones sobre tu atención médica antes, si así lo decides.
-Este programa incluye videos con información sobre cómo hacer un Poder Notarial para el Cuidado de la Salud. No tienes que verlos, pero pueden serte útiles.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if user_path == "Shirley":
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">[YOUTUBE 7qy101TRdiI]
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% elif user_path == "Frederico" or user_path == "Federico":
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">[YOUTUBE GR9t6ygX13g]
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% elif user_path == "Lisa":
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">[YOUTUBE h2ZGl568xHo]
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Para obtener más información, lee el artículo de ILAO sobre los [**Conceptos Básicos del Poder Notarial para el Cuidado de la Salud**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org/legal-information/setting-power-attorney-healthcare</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Después de descargar tus formularios, tendrás que firmar el documento frente a un testigo. El testigo también tendrá que firmar el documento. No necesitas saber quién será el testigo para usar este programa.
-Después de que el formulario esté firmado, querrás entregar copias del poder notarial a tu agente, así como a tus proveedores de atención médica. Tus formularios incluirán instrucciones con más información.
-Para obtener más información, lee el artículo de ILAO sobre los [**Conceptos Básicos del Poder Notarial para el Cuidado de la Salud**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org/legal-information/setting-power-attorney-healthcare</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>).
-Si deseas saber más sobre la planificación en caso de discapacidad o el cuidado al final de la vida, puedes revisar la guía de ILAO y CDEL [**Empodérate de tu Futuro**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ preview.url_for() }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Tu agente es una persona en quien confías y que eliges para tomar decisiones sobre tu atención médica y cuidado de tu salud por ti, si alguna vez necesitas ayuda. 
-Tu agente debe tener al menos 18 años de edad. Tu agente no tiene que ser un familiar, pero debe ser alguien en quien confíes. Tu agente no necesita ser ciudadano de los Estados Unidos. 
-Puedes seleccionar agentes sucesores como respaldo si el primer agente no puede tomar estas decisiones.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">${collapse_template(video_who_agent)}
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
- **Nota:** Si puedes comunicarte y entender tus opciones, tú eres quien toma las decisiones.
-Para obtener más información, lee el artículo de ILAO sobre [**Conceptos Básicos del Poder Notarial para el Cuidado de la Salud**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org/legal-information/setting-power-attorney-healthcare</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>No. Puedes nombrar como agente a alguien que vive fuera de los Estados Unidos. El agente no necesita ser ciudadano de los Estados Unidos. Sin embargo, pueden haber problemas si un banco u otra institución financiera no puede comunicarse con esa persona. Es posible que desees consultar a un abogado para obtener asesoramiento. Usa [**Obtener ayuda legal**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org/get-legal-help</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>) para encontrar servicios legales gratuitos o de bajo costo en tu área.
-Para direcciones internacionales, habrá espacio para ingresar la dirección en dos líneas. Debes escribir la dirección internacional usando el alfabeto inglés.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if for_yourself == True:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Puedes cambiar de opinión y poner fin a tu Poder Notarial para el Cuidado de la Salud en cualquier momento. Esto se llama revocación.
-La revocación significa que dejas de permitir que </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${agent.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> tome decisiones por ti. Para obtener más información, lee el artículo de ILAO sobre [**poner fin a un Poder Notarial**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org/legal-information/ending-power-attorney-0</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>).
-Puedes poner fin a un Poder Notarial haciendo una revocación formal. Para hacer una Revocación de Poder Notarial, usa el [**Formulario Guiado de Revocación de Poder Notarial**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org/legal-information/power-attorney-revocation</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">).
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${principal.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> puede cambiar de opinión y poner fin a su Poder Notarial para el Cuidado de la Salud en cualquier momento. Esto se llama revocación.
-La revocación significa que </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${principal.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> deja de permitir que </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${agent.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> tome decisiones en su nombre. Para obtener más información, lee el artículo de ILAO sobre [**poner fin a un Poder Notarial**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org/legal-information/ending-power-attorney-0</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">). 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${principal.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> puede poner fin a un Poder Notarial haciendo una revocación formal. Para hacer una Revocación de Poder Notarial, usa el [**Formulario Guiado de Revocación de Poder Notarial**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org/legal-information/power-attorney-revocation</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">).
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>% endif</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>No. Puedes nombrar como agente sucesor a alguien que vive fuera de los Estados Unidos. El agente sucesor no necesita ser ciudadano de los Estados Unidos. Sin embargo, puede haber problemas si un banco u otra institución financiera no puede comunicarse con esa persona. Es posible que desees consultar con un abogado. Usa [**Obtener ayuda legal**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org/get-legal-help</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>) para encontrar servicios legales gratuitos o de bajo costo en tu área.
-Para direcciones internacionales, habrá espacio para ingresar la dirección en dos líneas.
-Debes escribir la dirección internacional usando el alfabeto inglés.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Tus formularios están adjuntos.
-¡Gracias por usar los Formularios Guiados de ILAO!
-[Illinois Legal Aid Online](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">**Estás haciendo estos formularios para:**
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if for_yourself == True:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Para mí
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Para otra persona
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>% endif</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">**Your treatment instructions:**
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if quality_of_life == 'quality':
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The quality of my life is more important than the length of my life.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-% if quality_of_life == 'longevity':
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">I want my life to be prolonged to the greatest extent possible.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-% if quality_of_life == 'do_not':
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">I do not want to decide this now.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>**Tus instrucciones sobre tratamiento:**</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-% if quality_of_life == 'quality':
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">La calidad de mi vida es más importante que la duración de mi vida.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-% if quality_of_life == 'longevity':
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Quiero que mi vida se prolongue en la mayor medida posible.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-% if quality_of_life == 'do_not':
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">No quiero decidir esto ahora.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>% endif</t>
-    </r>
-  </si>
-  <si>
-    <t>docassemble.playground3PoAHealthCareSpanish:power_of_attorney_for_health_care.yml</t>
-  </si>
-  <si>
-    <t>64ed875eeb30496e64d73b9be2b5030e</t>
-  </si>
-  <si>
-    <t xml:space="preserve">About the witness
-</t>
-  </si>
-  <si>
-    <t>Acerca del testigo</t>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ action_button_html(interview_url(i="docassemble.ILAO:feedback.yml", easy_form_interview=ilao_easy_form_url, easy_form_title=ilao_easy_form_title, easy_form_page=current_context().question_id, easy_form_variable=current_context().variable, local=False,reset=1), label=':comment: ¿Fue útil este programa?', color="#181c36", size="md", new_window=True) }</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -23232,7 +23239,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H238"/>
+  <dimension ref="A1:H240"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="61.109375" customWidth="1"/>
@@ -23317,7 +23324,7 @@
         <v>16</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -23473,7 +23480,7 @@
         <v>33</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="28.8">
@@ -23487,7 +23494,7 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>11</v>
@@ -23496,7 +23503,7 @@
         <v>12</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>35</v>
@@ -23513,7 +23520,7 @@
         <v>1</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>11</v>
@@ -23522,7 +23529,7 @@
         <v>12</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>36</v>
@@ -23577,7 +23584,7 @@
         <v>42</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="28.8">
@@ -23681,7 +23688,7 @@
         <v>54</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="28.8">
@@ -23785,7 +23792,7 @@
         <v>66</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="57.6">
@@ -23811,7 +23818,7 @@
         <v>68</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="28.8">
@@ -23967,7 +23974,7 @@
         <v>82</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -24409,7 +24416,7 @@
         <v>125</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -24539,7 +24546,7 @@
         <v>136</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="28.8">
@@ -24565,7 +24572,7 @@
         <v>138</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="28.8">
@@ -24669,7 +24676,7 @@
         <v>149</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
     </row>
     <row r="56" spans="1:8" ht="28.8">
@@ -25007,7 +25014,7 @@
         <v>182</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="69" spans="1:8" ht="28.8">
@@ -25033,7 +25040,7 @@
         <v>184</v>
       </c>
       <c r="H69" s="9" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
     </row>
     <row r="70" spans="1:8">
@@ -25111,7 +25118,7 @@
         <v>190</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
     </row>
     <row r="73" spans="1:8">
@@ -25189,7 +25196,7 @@
         <v>198</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="76" spans="1:8" ht="115.2">
@@ -25241,7 +25248,7 @@
         <v>203</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
     </row>
     <row r="78" spans="1:8" ht="28.8">
@@ -25345,7 +25352,7 @@
         <v>213</v>
       </c>
       <c r="H81" s="3" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="82" spans="1:8">
@@ -25475,7 +25482,7 @@
         <v>226</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="87" spans="1:8" ht="43.2">
@@ -25527,7 +25534,7 @@
         <v>651</v>
       </c>
       <c r="H88" s="3" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="89" spans="1:8" ht="72">
@@ -25579,7 +25586,7 @@
         <v>234</v>
       </c>
       <c r="H90" s="3" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="91" spans="1:8">
@@ -25735,7 +25742,7 @@
         <v>249</v>
       </c>
       <c r="H96" s="6" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
     </row>
     <row r="97" spans="1:8" ht="129.6">
@@ -25761,7 +25768,7 @@
         <v>251</v>
       </c>
       <c r="H97" s="3" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="98" spans="1:8" ht="86.4">
@@ -25813,7 +25820,7 @@
         <v>256</v>
       </c>
       <c r="H99" s="3" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
     </row>
     <row r="100" spans="1:8" ht="28.8">
@@ -26096,7 +26103,7 @@
         <v>12</v>
       </c>
       <c r="G110" s="8" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="H110" s="3" t="s">
         <v>663</v>
@@ -26437,7 +26444,7 @@
         <v>313</v>
       </c>
       <c r="H123" s="8" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="124" spans="1:8" ht="28.8">
@@ -26463,7 +26470,7 @@
         <v>315</v>
       </c>
       <c r="H124" s="8" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="125" spans="1:8" ht="28.8">
@@ -26489,7 +26496,7 @@
         <v>317</v>
       </c>
       <c r="H125" s="8" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
     </row>
     <row r="126" spans="1:8">
@@ -26567,7 +26574,7 @@
         <v>324</v>
       </c>
       <c r="H128" s="3" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
     </row>
     <row r="129" spans="1:8">
@@ -26645,7 +26652,7 @@
         <v>331</v>
       </c>
       <c r="H131" s="3" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
     </row>
     <row r="132" spans="1:8">
@@ -26711,7 +26718,7 @@
         <v>2</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="E134" s="2" t="s">
         <v>11</v>
@@ -26720,10 +26727,10 @@
         <v>12</v>
       </c>
       <c r="G134" s="3" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="H134" s="3" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="135" spans="1:8" ht="409.6">
@@ -26749,7 +26756,7 @@
         <v>338</v>
       </c>
       <c r="H135" s="3" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
     </row>
     <row r="136" spans="1:8" ht="28.8">
@@ -26983,7 +26990,7 @@
         <v>360</v>
       </c>
       <c r="H144" s="3" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
     </row>
     <row r="145" spans="1:8">
@@ -27113,7 +27120,7 @@
         <v>374</v>
       </c>
       <c r="H149" s="3" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
     </row>
     <row r="150" spans="1:8" ht="28.8">
@@ -27243,7 +27250,7 @@
         <v>388</v>
       </c>
       <c r="H154" s="3" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
     </row>
     <row r="155" spans="1:8" ht="43.2">
@@ -27347,7 +27354,7 @@
         <v>400</v>
       </c>
       <c r="H158" s="6" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
     </row>
     <row r="159" spans="1:8" ht="100.8">
@@ -27399,7 +27406,7 @@
         <v>405</v>
       </c>
       <c r="H160" s="3" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
     </row>
     <row r="161" spans="1:8" ht="100.8">
@@ -27555,7 +27562,7 @@
         <v>423</v>
       </c>
       <c r="H166" s="3" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
     </row>
     <row r="167" spans="1:8" ht="57.6">
@@ -27711,7 +27718,7 @@
         <v>708</v>
       </c>
       <c r="H172" s="3" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
     </row>
     <row r="173" spans="1:8" ht="28.8">
@@ -27760,10 +27767,10 @@
         <v>12</v>
       </c>
       <c r="G174" s="3" t="s">
-        <v>775</v>
+        <v>789</v>
       </c>
       <c r="H174" s="3" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
     </row>
     <row r="175" spans="1:8" ht="201.6">
@@ -27789,7 +27796,7 @@
         <v>446</v>
       </c>
       <c r="H175" s="3" t="s">
-        <v>709</v>
+        <v>790</v>
       </c>
     </row>
     <row r="176" spans="1:8" ht="86.4">
@@ -27815,7 +27822,7 @@
         <v>449</v>
       </c>
       <c r="H176" s="3" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
     </row>
     <row r="177" spans="1:8">
@@ -27867,7 +27874,7 @@
         <v>455</v>
       </c>
       <c r="H178" s="6" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
     </row>
     <row r="179" spans="1:8">
@@ -27893,7 +27900,7 @@
         <v>458</v>
       </c>
       <c r="H179" s="6" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
     </row>
     <row r="180" spans="1:8">
@@ -27919,7 +27926,7 @@
         <v>461</v>
       </c>
       <c r="H180" s="6" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="181" spans="1:8">
@@ -27945,7 +27952,7 @@
         <v>464</v>
       </c>
       <c r="H181" s="6" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
     </row>
     <row r="182" spans="1:8">
@@ -27971,7 +27978,7 @@
         <v>467</v>
       </c>
       <c r="H182" s="6" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
     </row>
     <row r="183" spans="1:8" ht="144">
@@ -27997,7 +28004,7 @@
         <v>470</v>
       </c>
       <c r="H183" s="3" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="184" spans="1:8" ht="28.8">
@@ -28231,7 +28238,7 @@
         <v>496</v>
       </c>
       <c r="H192" s="6" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
     </row>
     <row r="193" spans="1:8">
@@ -28309,7 +28316,7 @@
         <v>504</v>
       </c>
       <c r="H195" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
     </row>
     <row r="196" spans="1:8">
@@ -28335,7 +28342,7 @@
         <v>506</v>
       </c>
       <c r="H196" s="6" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
     </row>
     <row r="197" spans="1:8" ht="100.8">
@@ -28361,7 +28368,7 @@
         <v>508</v>
       </c>
       <c r="H197" s="3" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
     </row>
     <row r="198" spans="1:8" ht="158.4">
@@ -28387,7 +28394,7 @@
         <v>510</v>
       </c>
       <c r="H198" s="3" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="199" spans="1:8" ht="43.2">
@@ -28413,7 +28420,7 @@
         <v>512</v>
       </c>
       <c r="H199" s="3" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="200" spans="1:8" ht="100.8">
@@ -28439,7 +28446,7 @@
         <v>514</v>
       </c>
       <c r="H200" s="3" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="201" spans="1:8" ht="43.2">
@@ -28465,7 +28472,7 @@
         <v>516</v>
       </c>
       <c r="H201" s="3" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="202" spans="1:8" ht="100.8">
@@ -28491,7 +28498,7 @@
         <v>518</v>
       </c>
       <c r="H202" s="3" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
     </row>
     <row r="203" spans="1:8" ht="100.8">
@@ -28517,7 +28524,7 @@
         <v>520</v>
       </c>
       <c r="H203" s="3" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
     </row>
     <row r="204" spans="1:8" ht="115.2">
@@ -28543,7 +28550,7 @@
         <v>522</v>
       </c>
       <c r="H204" s="3" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="205" spans="1:8" ht="158.4">
@@ -28569,7 +28576,7 @@
         <v>524</v>
       </c>
       <c r="H205" s="3" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="206" spans="1:8" ht="172.8">
@@ -28595,7 +28602,7 @@
         <v>526</v>
       </c>
       <c r="H206" s="3" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="207" spans="1:8" ht="115.2">
@@ -28621,7 +28628,7 @@
         <v>528</v>
       </c>
       <c r="H207" s="3" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="208" spans="1:8" ht="158.4">
@@ -28644,10 +28651,10 @@
         <v>12</v>
       </c>
       <c r="G208" s="3" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="H208" s="3" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
     </row>
     <row r="209" spans="1:8" ht="158.4">
@@ -28673,7 +28680,7 @@
         <v>531</v>
       </c>
       <c r="H209" s="3" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="210" spans="1:8" ht="100.8">
@@ -28699,7 +28706,7 @@
         <v>533</v>
       </c>
       <c r="H210" s="3" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
     </row>
     <row r="211" spans="1:8" ht="100.8">
@@ -28725,7 +28732,7 @@
         <v>535</v>
       </c>
       <c r="H211" s="3" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
     </row>
     <row r="212" spans="1:8" ht="43.2">
@@ -28751,7 +28758,7 @@
         <v>537</v>
       </c>
       <c r="H212" s="3" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
     </row>
     <row r="213" spans="1:8" ht="43.2">
@@ -28803,7 +28810,7 @@
         <v>542</v>
       </c>
       <c r="H214" s="3" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
     </row>
     <row r="215" spans="1:8" ht="288">
@@ -28829,7 +28836,7 @@
         <v>544</v>
       </c>
       <c r="H215" s="3" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
     </row>
     <row r="216" spans="1:8" ht="115.2">
@@ -28855,7 +28862,7 @@
         <v>546</v>
       </c>
       <c r="H216" s="3" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
     </row>
     <row r="217" spans="1:8" ht="43.2">
@@ -28985,7 +28992,7 @@
         <v>557</v>
       </c>
       <c r="H221" s="3" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
     </row>
     <row r="222" spans="1:8" ht="43.2">
@@ -29406,7 +29413,7 @@
     </row>
     <row r="238" spans="1:8">
       <c r="A238" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
       <c r="B238" t="s">
         <v>599</v>
@@ -29415,7 +29422,7 @@
         <v>1</v>
       </c>
       <c r="D238" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
       <c r="E238" t="s">
         <v>11</v>
@@ -29424,11 +29431,31 @@
         <v>12</v>
       </c>
       <c r="G238" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="H238" s="4" t="s">
-        <v>790</v>
-      </c>
+        <v>788</v>
+      </c>
+    </row>
+    <row r="239" spans="1:8">
+      <c r="A239" s="2"/>
+      <c r="B239" s="2"/>
+      <c r="C239" s="2"/>
+      <c r="D239" s="2"/>
+      <c r="E239" s="2"/>
+      <c r="F239" s="2"/>
+      <c r="G239" s="3"/>
+      <c r="H239" s="3"/>
+    </row>
+    <row r="240" spans="1:8">
+      <c r="A240" s="2"/>
+      <c r="B240" s="2"/>
+      <c r="C240" s="2"/>
+      <c r="D240" s="2"/>
+      <c r="E240" s="2"/>
+      <c r="F240" s="2"/>
+      <c r="G240" s="3"/>
+      <c r="H240" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
get docs screen translation now active
</commit_message>
<xml_diff>
--- a/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
+++ b/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4D47FC-559F-467F-9C85-E42AD8F50C3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6134A77E-A56B-4A08-AD08-7A572988C9E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-34545" yWindow="-1995" windowWidth="30045" windowHeight="19425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-32055" yWindow="645" windowWidth="19530" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22005,214 +22005,6 @@
   <si>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Your forms are ready. View and download your forms below. Click **Make changes** to fix any mistakes.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if user_path == "Shirley":
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[YOUTUBE NE0faXuz5v4]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% elif user_path == "Frederico" or user_path == "Federico":
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[YOUTUBE g5Vdv0hWJ6g]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% elif user_path == "Lisa":
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[YOUTUBE F2QbdrhcZ0g]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Read the instructions to learn what to do next.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ action_button_html(url_action('review_answers'), label='^^edit^^ Make changes', color='success', size="md") }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ al_user_bundle.download_list_html() }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-&amp;nbsp;
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ al_user_bundle.send_button_html(show_editable_checkbox=False) }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-**Note:** The Power of Attorney needs to be signed in front of at least one witness to become official.
-Thank you for using ILAO Easy Forms!
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
         <b/>
         <sz val="11"/>
         <color rgb="FF008000"/>
@@ -22847,6 +22639,206 @@
       <t xml:space="preserve">
 **Nota:** El Poder Notarial debe firmarse frente a al menos un testigo para que sea válido.
 ¡Gracias por usar los Formularios Guiados de ILAO!</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Your forms are ready. View and download your forms below. Click **Make changes** to fix any mistakes.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if user_path == "Shirley":
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[YOUTUBE NE0faXuz5v4]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% elif user_path == "Frederico" or user_path == "Federico":
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[YOUTUBE g5Vdv0hWJ6g]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% elif user_path == "Lisa":
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[YOUTUBE F2QbdrhcZ0g]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Read the instructions to learn what to do next.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ action_button_html(url_action('review_answers'), label=':edit: Make changes', color='success', size='md') }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ al_user_bundle.download_list_html(view_label='View', download_label='Download', zip_label='Download all') }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ al_user_bundle.send_button_html(show_editable_checkbox=False, label='Send') }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+**Note:** The Power of Attorney needs to be signed in front of at least one witness to become official.
+Thank you for using ILAO Easy Forms!
+</t>
     </r>
   </si>
 </sst>
@@ -23397,7 +23389,7 @@
         <v>16</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -23709,7 +23701,7 @@
         <v>48</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="28.8">
@@ -23769,13 +23761,13 @@
         <v>781</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="C18" s="2">
         <v>0</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>11</v>
@@ -23784,10 +23776,10 @@
         <v>12</v>
       </c>
       <c r="G18" s="3" t="s">
+        <v>790</v>
+      </c>
+      <c r="H18" s="3" t="s">
         <v>791</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>792</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="28.8">
@@ -23795,7 +23787,7 @@
         <v>781</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="C19" s="2">
         <v>1</v>
@@ -26837,13 +26829,13 @@
         <v>781</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="C136" s="2">
         <v>0</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="E136" s="2" t="s">
         <v>11</v>
@@ -26852,10 +26844,10 @@
         <v>12</v>
       </c>
       <c r="G136" s="3" t="s">
+        <v>794</v>
+      </c>
+      <c r="H136" s="3" t="s">
         <v>795</v>
-      </c>
-      <c r="H136" s="3" t="s">
-        <v>796</v>
       </c>
     </row>
     <row r="137" spans="1:8" ht="409.6">
@@ -27872,7 +27864,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="176" spans="1:8" ht="388.8">
+    <row r="176" spans="1:8" ht="374.4">
       <c r="A176" s="2" t="s">
         <v>8</v>
       </c>
@@ -27892,10 +27884,10 @@
         <v>12</v>
       </c>
       <c r="G176" s="3" t="s">
-        <v>785</v>
+        <v>797</v>
       </c>
       <c r="H176" s="3" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
     </row>
     <row r="177" spans="1:8" ht="201.6">
@@ -27921,7 +27913,7 @@
         <v>445</v>
       </c>
       <c r="H177" s="3" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
     </row>
     <row r="178" spans="1:8" ht="86.4">

</xml_diff>

<commit_message>
added instructions and fixed question and field translations
</commit_message>
<xml_diff>
--- a/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
+++ b/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24235661-ED45-4127-BBDE-4E397A8609F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB43FF36-A6FE-43D2-B494-EFFC05E36C46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5340" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20391,63 +20391,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Después de descargar tus formularios, tendrás que firmar el documento frente a un testigo. El testigo también tendrá que firmar el documento. No necesitas saber quién será el testigo para usar este programa.
-Después de que el formulario esté firmado, querrás entregar copias del poder notarial a tu agente, así como a tus proveedores de atención médica. Tus formularios incluirán instrucciones con más información.
-Para obtener más información, lee el artículo de ILAO sobre los [**Conceptos Básicos del Poder Notarial para el Cuidado de la Salud**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org/legal-information/setting-power-attorney-healthcare</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>).
-Si deseas saber más sobre la planificación en caso de discapacidad o el cuidado al final de la vida, puedes revisar la guía de ILAO y CDEL [**Empodérate de tu Futuro**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ preview.url_for() }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
       <t xml:space="preserve">Tu agente es una persona en quien confías y que eliges para tomar decisiones sobre tu atención médica y cuidado de tu salud por ti, si alguna vez necesitas ayuda. 
 Tu agente debe tener al menos 18 años de edad. Tu agente no tiene que ser un familiar, pero debe ser alguien en quien confíes. Tu agente no necesita ser ciudadano de los Estados Unidos. 
 Puedes seleccionar agentes sucesores como respaldo si el primer agente no puede tomar estas decisiones.
@@ -22832,6 +22775,63 @@
         <scheme val="minor"/>
       </rPr>
       <t>${collapse_template(video_cooling)}</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Después de descargar tus formularios, tendrás que firmar el documento frente a un testigo. El testigo también tendrá que firmar el documento. No necesitas saber quién será el testigo para usar este programa.
+Después de que el formulario esté firmado, querrás entregar copias del poder notarial a tu agente, así como a tus proveedores de atención médica. Tus formularios incluirán instrucciones con más información.
+Para obtener más información, lee el artículo de ILAO sobre los [**Conceptos Básicos del Poder Notarial para el Cuidado de la Salud**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/legal-information/setting-power-attorney-healthcare</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).
+Si deseas saber más sobre la planificación en caso de discapacidad o el cuidado al final de la vida, puedes revisar la guía de ILAO y CDEL [**Empodérate de tu Futuro**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ preview_es.url_for() }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).</t>
     </r>
   </si>
 </sst>
@@ -23382,7 +23382,7 @@
         <v>16</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -23642,7 +23642,7 @@
         <v>42</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>763</v>
+        <v>797</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="28.8">
@@ -23694,7 +23694,7 @@
         <v>48</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="28.8">
@@ -23746,21 +23746,21 @@
         <v>54</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="115.2">
       <c r="A18" s="2" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="C18" s="2">
         <v>0</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>11</v>
@@ -23769,18 +23769,18 @@
         <v>12</v>
       </c>
       <c r="G18" s="3" t="s">
+        <v>779</v>
+      </c>
+      <c r="H18" s="3" t="s">
         <v>780</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>781</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="28.8">
       <c r="A19" s="2" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="C19" s="2">
         <v>1</v>
@@ -24046,7 +24046,7 @@
         <v>1</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>11</v>
@@ -24055,10 +24055,10 @@
         <v>12</v>
       </c>
       <c r="G29" s="3" t="s">
+        <v>792</v>
+      </c>
+      <c r="H29" s="3" t="s">
         <v>793</v>
-      </c>
-      <c r="H29" s="3" t="s">
-        <v>794</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -24162,7 +24162,7 @@
         <v>87</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -24630,7 +24630,7 @@
         <v>133</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="28.8">
@@ -24734,7 +24734,7 @@
         <v>144</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
     </row>
     <row r="56" spans="1:8" ht="288">
@@ -25381,7 +25381,7 @@
         <v>12</v>
       </c>
       <c r="G80" s="3" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="H80" s="3" t="s">
         <v>639</v>
@@ -25852,7 +25852,7 @@
         <v>247</v>
       </c>
       <c r="H98" s="3" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
     </row>
     <row r="99" spans="1:8" ht="86.4">
@@ -26736,7 +26736,7 @@
         <v>327</v>
       </c>
       <c r="H132" s="3" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="133" spans="1:8">
@@ -26819,16 +26819,16 @@
     </row>
     <row r="136" spans="1:8" ht="115.2">
       <c r="A136" s="2" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="C136" s="2">
         <v>0</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="E136" s="2" t="s">
         <v>11</v>
@@ -26837,10 +26837,10 @@
         <v>12</v>
       </c>
       <c r="G136" s="3" t="s">
+        <v>783</v>
+      </c>
+      <c r="H136" s="3" t="s">
         <v>784</v>
-      </c>
-      <c r="H136" s="3" t="s">
-        <v>785</v>
       </c>
     </row>
     <row r="137" spans="1:8" ht="409.6">
@@ -26866,7 +26866,7 @@
         <v>334</v>
       </c>
       <c r="H137" s="3" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
     </row>
     <row r="138" spans="1:8" ht="28.8">
@@ -27100,7 +27100,7 @@
         <v>356</v>
       </c>
       <c r="H146" s="3" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
     </row>
     <row r="147" spans="1:8">
@@ -27230,7 +27230,7 @@
         <v>370</v>
       </c>
       <c r="H151" s="3" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
     </row>
     <row r="152" spans="1:8" ht="28.8">
@@ -27877,10 +27877,10 @@
         <v>12</v>
       </c>
       <c r="G176" s="3" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="H176" s="3" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
     </row>
     <row r="177" spans="1:8" ht="201.6">
@@ -27906,7 +27906,7 @@
         <v>442</v>
       </c>
       <c r="H177" s="3" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
     </row>
     <row r="178" spans="1:8" ht="86.4">
@@ -27932,7 +27932,7 @@
         <v>445</v>
       </c>
       <c r="H178" s="3" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
     </row>
     <row r="179" spans="1:8">
@@ -28478,7 +28478,7 @@
         <v>504</v>
       </c>
       <c r="H199" s="3" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
     </row>
     <row r="200" spans="1:8" ht="158.4">
@@ -28761,10 +28761,10 @@
         <v>12</v>
       </c>
       <c r="G210" s="3" t="s">
+        <v>769</v>
+      </c>
+      <c r="H210" s="3" t="s">
         <v>770</v>
-      </c>
-      <c r="H210" s="3" t="s">
-        <v>771</v>
       </c>
     </row>
     <row r="211" spans="1:8" ht="158.4">
@@ -29523,7 +29523,7 @@
     </row>
     <row r="240" spans="1:8">
       <c r="A240" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="B240" t="s">
         <v>595</v>
@@ -29532,7 +29532,7 @@
         <v>1</v>
       </c>
       <c r="D240" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="E240" t="s">
         <v>11</v>
@@ -29541,10 +29541,10 @@
         <v>12</v>
       </c>
       <c r="G240" t="s">
+        <v>773</v>
+      </c>
+      <c r="H240" s="4" t="s">
         <v>774</v>
-      </c>
-      <c r="H240" s="4" t="s">
-        <v>775</v>
       </c>
     </row>
     <row r="241" spans="1:8">

</xml_diff>

<commit_message>
translation improvements to interview and review screens
</commit_message>
<xml_diff>
--- a/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
+++ b/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB43FF36-A6FE-43D2-B494-EFFC05E36C46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCD8239A-22B3-4E79-9362-9091D3D53A3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5340" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-34695" yWindow="-2895" windowWidth="31785" windowHeight="17910" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -10524,386 +10524,6 @@
     </r>
   </si>
   <si>
-    <t>4df62dd05d59a5e95853014f178b6ac4</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">**Limits for </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${agent.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">:**
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if limit_checkboxes['no_autopsy']:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">* </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${subject_do_does}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> not authorize an autopsy.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if limit_checkboxes['no_science']:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">* </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${subject_do_does}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> not authorize donation of </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${my_their}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> remains to science.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if limit_checkboxes['no_start']:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">* </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${subject_do_does}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> not authorize starting these treatments: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${fix_punctuation(no_start_text)}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if limit_checkboxes['no_end']:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">* </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${subject_do_does}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> not authorize ending these treatments: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${fix_punctuation(no_end_text)}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if limit_checkboxes['other']:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">* </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${fix_punctuation(other_limits)}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-  </si>
-  <si>
     <t>53f4eea875cd986be67631969353d829</t>
   </si>
   <si>
@@ -17277,338 +16897,6 @@
   <si>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">**Límites para </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${agent.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">:**
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if limit_checkboxes['no_autopsy']:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">* </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${subject_do_does}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> no autoriza una autopsia.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-% if limit_checkboxes['no_science']:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">* </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${subject_do_does}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> no autoriza la donación de </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${my_their}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> restos a la ciencia.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-% if limit_checkboxes['no_start']:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">* </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${subject_do_does}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> no autoriza iniciar estos tratamientos: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${fix_punctuation(no_start_text)}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-% if limit_checkboxes['no_end']:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">* </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${subject_do_does}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> no autoriza suspender estos tratamientos: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${fix_punctuation(no_end_text)}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-% if limit_checkboxes['other']:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">* </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${fix_punctuation(other_limits)}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>% endif</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
         <b/>
         <sz val="11"/>
         <color rgb="FF008000"/>
@@ -22832,6 +22120,990 @@
         <scheme val="minor"/>
       </rPr>
       <t>).</t>
+    </r>
+  </si>
+  <si>
+    <t>98dc4f5f71b807757f3e798f7c664c92</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">**Limits for </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${agent.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">:**
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if limit_checkboxes['no_autopsy'] and for_yourself:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* I do not authorize an autopsy.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if limit_checkboxes['no_science'] and for_yourself:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* I do not authorize donation of my remains to science.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if limit_checkboxes['no_start'] and for_yourself:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* I do not authorize starting these treatments: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${fix_punctuation(no_start_text)}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if limit_checkboxes['no_end'] and for_yourself:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* I do not authorize ending these treatments: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${fix_punctuation(no_end_text)}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if limit_checkboxes['no_autopsy'] and not for_yourself:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> does not authorize an autopsy.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if limit_checkboxes['no_science'] and not for_yourself:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> does not authorize donation of their remains to science.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if limit_checkboxes['no_start'] and not for_yourself:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> does not authorize starting these treatments: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${fix_punctuation(no_start_text)}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if limit_checkboxes['no_end'] and not for_yourself:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> does not authorize ending these treatments: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${fix_punctuation(no_end_text)}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if limit_checkboxes['other']:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${fix_punctuation(other_limits)}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">**Límites para </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${agent.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">:**
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if limit_checkboxes['no_autopsy'] and for_yourself:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* Yo no autorizo una autopsia.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+% if limit_checkboxes['no_science'] and for_yourself:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* Yo no autorizo la donación de mi restos a la ciencia.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+% if limit_checkboxes['no_start'] and for_yourself:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* Yo no autorizo iniciar estos tratamientos: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${fix_punctuation(no_start_text)}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+% if limit_checkboxes['no_end'] and for_yourself:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* Yo no autorizo suspender estos tratamientos: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${fix_punctuation(no_end_text)}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+% if limit_checkboxes['no_autopsy'] and not for_yourself:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> no autoriza una autopsia.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+% if limit_checkboxes['no_science'] and not for_yourself:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> no autoriza la donación de sus restos a la ciencia.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+% if limit_checkboxes['no_start'] and not for_yourself:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> no autoriza iniciar estos tratamientos: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${fix_punctuation(no_start_text)}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+% if limit_checkboxes['no_end'] and not for_yourself:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> no autoriza suspender estos tratamientos: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${fix_punctuation(no_end_text)}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+% if limit_checkboxes['other']:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${fix_punctuation(other_limits)}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
     </r>
   </si>
 </sst>
@@ -23297,7 +23569,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H242"/>
+  <dimension ref="A1:I242"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="61.109375" customWidth="1"/>
@@ -23305,6 +23577,7 @@
     <col min="3" max="3" width="12.6640625" customWidth="1"/>
     <col min="4" max="4" width="32.5546875" customWidth="1"/>
     <col min="7" max="8" width="75.6640625" customWidth="1"/>
+    <col min="9" max="9" width="15.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -23382,7 +23655,7 @@
         <v>16</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>787</v>
+        <v>784</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -23434,7 +23707,7 @@
         <v>22</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -23538,7 +23811,7 @@
         <v>33</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>752</v>
+        <v>749</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="28.8">
@@ -23552,7 +23825,7 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>11</v>
@@ -23561,7 +23834,7 @@
         <v>12</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>760</v>
+        <v>757</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>35</v>
@@ -23578,7 +23851,7 @@
         <v>1</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>758</v>
+        <v>755</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>11</v>
@@ -23587,7 +23860,7 @@
         <v>12</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>759</v>
+        <v>756</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>36</v>
@@ -23642,7 +23915,7 @@
         <v>42</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="28.8">
@@ -23694,7 +23967,7 @@
         <v>48</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>776</v>
+        <v>773</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="28.8">
@@ -23746,21 +24019,21 @@
         <v>54</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>763</v>
+        <v>760</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="115.2">
       <c r="A18" s="2" t="s">
-        <v>771</v>
+        <v>768</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>777</v>
+        <v>774</v>
       </c>
       <c r="C18" s="2">
         <v>0</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>778</v>
+        <v>775</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>11</v>
@@ -23769,18 +24042,18 @@
         <v>12</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="28.8">
       <c r="A19" s="2" t="s">
-        <v>771</v>
+        <v>768</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>777</v>
+        <v>774</v>
       </c>
       <c r="C19" s="2">
         <v>1</v>
@@ -23824,7 +24097,7 @@
         <v>60</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -23850,7 +24123,7 @@
         <v>63</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="43.2">
@@ -23876,7 +24149,7 @@
         <v>65</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>753</v>
+        <v>750</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="57.6">
@@ -23902,7 +24175,7 @@
         <v>67</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="28.8">
@@ -23928,7 +24201,7 @@
         <v>69</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="57.6">
@@ -23954,7 +24227,7 @@
         <v>71</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="28.8">
@@ -23980,7 +24253,7 @@
         <v>74</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="244.8">
@@ -24006,7 +24279,7 @@
         <v>76</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="86.4">
@@ -24032,7 +24305,7 @@
         <v>79</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="409.6">
@@ -24046,7 +24319,7 @@
         <v>1</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>11</v>
@@ -24055,10 +24328,10 @@
         <v>12</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -24084,7 +24357,7 @@
         <v>81</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -24110,7 +24383,7 @@
         <v>83</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -24136,7 +24409,7 @@
         <v>85</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -24162,7 +24435,7 @@
         <v>87</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>788</v>
+        <v>785</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -24214,7 +24487,7 @@
         <v>92</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="100.8">
@@ -24240,7 +24513,7 @@
         <v>95</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="28.8">
@@ -24266,7 +24539,7 @@
         <v>97</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="86.4">
@@ -24292,7 +24565,7 @@
         <v>100</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="28.8">
@@ -24318,7 +24591,7 @@
         <v>103</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="144">
@@ -24344,7 +24617,7 @@
         <v>105</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="86.4">
@@ -24396,7 +24669,7 @@
         <v>112</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="374.4">
@@ -24422,7 +24695,7 @@
         <v>114</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="86.4">
@@ -24448,7 +24721,7 @@
         <v>117</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="28.8">
@@ -24474,7 +24747,7 @@
         <v>119</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="28.8">
@@ -24500,7 +24773,7 @@
         <v>122</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -24526,7 +24799,7 @@
         <v>124</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="43.2">
@@ -24552,7 +24825,7 @@
         <v>126</v>
       </c>
       <c r="H48" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -24578,7 +24851,7 @@
         <v>128</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -24604,7 +24877,7 @@
         <v>130</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="129.6">
@@ -24630,7 +24903,7 @@
         <v>133</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>764</v>
+        <v>761</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="28.8">
@@ -24656,7 +24929,7 @@
         <v>135</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="28.8">
@@ -24708,7 +24981,7 @@
         <v>141</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
     </row>
     <row r="55" spans="1:8" ht="100.8">
@@ -24734,7 +25007,7 @@
         <v>144</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
     </row>
     <row r="56" spans="1:8" ht="288">
@@ -24760,7 +25033,7 @@
         <v>146</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="28.8">
@@ -24786,7 +25059,7 @@
         <v>149</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -24838,7 +25111,7 @@
         <v>155</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
     </row>
     <row r="60" spans="1:8" ht="28.8">
@@ -24864,7 +25137,7 @@
         <v>157</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
     </row>
     <row r="61" spans="1:8" ht="144">
@@ -24890,7 +25163,7 @@
         <v>159</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -24968,7 +25241,7 @@
         <v>167</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
     </row>
     <row r="65" spans="1:8" ht="43.2">
@@ -24994,7 +25267,7 @@
         <v>169</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="57.6">
@@ -25020,7 +25293,7 @@
         <v>171</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
     </row>
     <row r="67" spans="1:8">
@@ -25072,7 +25345,7 @@
         <v>177</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
     </row>
     <row r="69" spans="1:8" ht="172.8">
@@ -25098,7 +25371,7 @@
         <v>179</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
     </row>
     <row r="70" spans="1:8" ht="28.8">
@@ -25124,7 +25397,7 @@
         <v>181</v>
       </c>
       <c r="H70" s="9" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
     </row>
     <row r="71" spans="1:8">
@@ -25150,7 +25423,7 @@
         <v>183</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
     </row>
     <row r="72" spans="1:8" ht="43.2">
@@ -25176,7 +25449,7 @@
         <v>185</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
     </row>
     <row r="73" spans="1:8" ht="57.6">
@@ -25202,7 +25475,7 @@
         <v>187</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -25228,7 +25501,7 @@
         <v>189</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="28.8">
@@ -25280,7 +25553,7 @@
         <v>195</v>
       </c>
       <c r="H76" s="3" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
     </row>
     <row r="77" spans="1:8" ht="115.2">
@@ -25306,7 +25579,7 @@
         <v>198</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
     </row>
     <row r="78" spans="1:8" ht="360">
@@ -25332,7 +25605,7 @@
         <v>200</v>
       </c>
       <c r="H78" s="3" t="s">
-        <v>731</v>
+        <v>728</v>
       </c>
     </row>
     <row r="79" spans="1:8" ht="28.8">
@@ -25358,7 +25631,7 @@
         <v>203</v>
       </c>
       <c r="H79" s="6" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
     </row>
     <row r="80" spans="1:8" ht="28.8">
@@ -25381,10 +25654,10 @@
         <v>12</v>
       </c>
       <c r="G80" s="3" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
     </row>
     <row r="81" spans="1:8" ht="72">
@@ -25410,7 +25683,7 @@
         <v>207</v>
       </c>
       <c r="H81" s="3" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
     </row>
     <row r="82" spans="1:8" ht="72">
@@ -25436,7 +25709,7 @@
         <v>209</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>732</v>
+        <v>729</v>
       </c>
     </row>
     <row r="83" spans="1:8">
@@ -25488,7 +25761,7 @@
         <v>214</v>
       </c>
       <c r="H84" s="3" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
     </row>
     <row r="85" spans="1:8">
@@ -25514,7 +25787,7 @@
         <v>216</v>
       </c>
       <c r="H85" s="6" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
     </row>
     <row r="86" spans="1:8">
@@ -25566,7 +25839,7 @@
         <v>222</v>
       </c>
       <c r="H87" s="6" t="s">
-        <v>733</v>
+        <v>730</v>
       </c>
     </row>
     <row r="88" spans="1:8" ht="43.2">
@@ -25592,7 +25865,7 @@
         <v>224</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
     </row>
     <row r="89" spans="1:8" ht="43.2">
@@ -25615,10 +25888,10 @@
         <v>12</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="H89" s="3" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
     </row>
     <row r="90" spans="1:8" ht="72">
@@ -25644,7 +25917,7 @@
         <v>228</v>
       </c>
       <c r="H90" s="3" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
     </row>
     <row r="91" spans="1:8" ht="72">
@@ -25670,7 +25943,7 @@
         <v>230</v>
       </c>
       <c r="H91" s="3" t="s">
-        <v>735</v>
+        <v>732</v>
       </c>
     </row>
     <row r="92" spans="1:8">
@@ -25722,7 +25995,7 @@
         <v>235</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
     </row>
     <row r="94" spans="1:8">
@@ -25748,7 +26021,7 @@
         <v>237</v>
       </c>
       <c r="H94" s="6" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
     </row>
     <row r="95" spans="1:8">
@@ -25774,7 +26047,7 @@
         <v>239</v>
       </c>
       <c r="H95" s="6" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
     </row>
     <row r="96" spans="1:8" ht="201.6">
@@ -25800,7 +26073,7 @@
         <v>242</v>
       </c>
       <c r="H96" s="3" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
     </row>
     <row r="97" spans="1:8" ht="28.8">
@@ -25826,7 +26099,7 @@
         <v>245</v>
       </c>
       <c r="H97" s="6" t="s">
-        <v>736</v>
+        <v>733</v>
       </c>
     </row>
     <row r="98" spans="1:8" ht="129.6">
@@ -25852,7 +26125,7 @@
         <v>247</v>
       </c>
       <c r="H98" s="3" t="s">
-        <v>795</v>
+        <v>792</v>
       </c>
     </row>
     <row r="99" spans="1:8" ht="86.4">
@@ -25878,7 +26151,7 @@
         <v>250</v>
       </c>
       <c r="H99" s="3" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
     </row>
     <row r="100" spans="1:8" ht="302.39999999999998">
@@ -25904,7 +26177,7 @@
         <v>252</v>
       </c>
       <c r="H100" s="3" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
     </row>
     <row r="101" spans="1:8" ht="28.8">
@@ -25930,7 +26203,7 @@
         <v>255</v>
       </c>
       <c r="H101" s="3" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
     </row>
     <row r="102" spans="1:8" ht="86.4">
@@ -25956,7 +26229,7 @@
         <v>257</v>
       </c>
       <c r="H102" s="3" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
     </row>
     <row r="103" spans="1:8">
@@ -26008,7 +26281,7 @@
         <v>262</v>
       </c>
       <c r="H104" s="6" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
     </row>
     <row r="105" spans="1:8">
@@ -26060,7 +26333,7 @@
         <v>267</v>
       </c>
       <c r="H106" s="6" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
     </row>
     <row r="107" spans="1:8">
@@ -26138,7 +26411,7 @@
         <v>275</v>
       </c>
       <c r="H109" s="6" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
     </row>
     <row r="110" spans="1:8" ht="43.2">
@@ -26164,7 +26437,7 @@
         <v>278</v>
       </c>
       <c r="H110" s="3" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
     </row>
     <row r="111" spans="1:8" ht="86.4">
@@ -26187,10 +26460,10 @@
         <v>12</v>
       </c>
       <c r="G111" s="8" t="s">
-        <v>750</v>
+        <v>747</v>
       </c>
       <c r="H111" s="3" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
     </row>
     <row r="112" spans="1:8">
@@ -26216,7 +26489,7 @@
         <v>281</v>
       </c>
       <c r="H112" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
     </row>
     <row r="113" spans="1:8">
@@ -26242,7 +26515,7 @@
         <v>283</v>
       </c>
       <c r="H113" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
     </row>
     <row r="114" spans="1:8">
@@ -26268,7 +26541,7 @@
         <v>285</v>
       </c>
       <c r="H114" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
     </row>
     <row r="115" spans="1:8">
@@ -26294,7 +26567,7 @@
         <v>287</v>
       </c>
       <c r="H115" s="6" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
     </row>
     <row r="116" spans="1:8" ht="43.2">
@@ -26320,7 +26593,7 @@
         <v>289</v>
       </c>
       <c r="H116" s="6" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
     </row>
     <row r="117" spans="1:8" ht="28.8">
@@ -26398,7 +26671,7 @@
         <v>297</v>
       </c>
       <c r="H119" s="6" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
     </row>
     <row r="120" spans="1:8" ht="28.8">
@@ -26424,7 +26697,7 @@
         <v>300</v>
       </c>
       <c r="H120" s="3" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
     </row>
     <row r="121" spans="1:8">
@@ -26450,7 +26723,7 @@
         <v>302</v>
       </c>
       <c r="H121" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
     </row>
     <row r="122" spans="1:8" ht="86.4">
@@ -26476,7 +26749,7 @@
         <v>305</v>
       </c>
       <c r="H122" s="3" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
     </row>
     <row r="123" spans="1:8" ht="28.8">
@@ -26502,7 +26775,7 @@
         <v>307</v>
       </c>
       <c r="H123" s="6" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
     </row>
     <row r="124" spans="1:8" ht="28.8">
@@ -26528,7 +26801,7 @@
         <v>309</v>
       </c>
       <c r="H124" s="8" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
     </row>
     <row r="125" spans="1:8" ht="28.8">
@@ -26554,7 +26827,7 @@
         <v>311</v>
       </c>
       <c r="H125" s="8" t="s">
-        <v>751</v>
+        <v>748</v>
       </c>
     </row>
     <row r="126" spans="1:8" ht="28.8">
@@ -26580,7 +26853,7 @@
         <v>313</v>
       </c>
       <c r="H126" s="8" t="s">
-        <v>739</v>
+        <v>736</v>
       </c>
     </row>
     <row r="127" spans="1:8">
@@ -26606,7 +26879,7 @@
         <v>315</v>
       </c>
       <c r="H127" s="8" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
     </row>
     <row r="128" spans="1:8">
@@ -26658,7 +26931,7 @@
         <v>320</v>
       </c>
       <c r="H129" s="3" t="s">
-        <v>737</v>
+        <v>734</v>
       </c>
     </row>
     <row r="130" spans="1:8">
@@ -26684,7 +26957,7 @@
         <v>322</v>
       </c>
       <c r="H130" s="3" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
     </row>
     <row r="131" spans="1:8" ht="28.8">
@@ -26710,7 +26983,7 @@
         <v>325</v>
       </c>
       <c r="H131" s="6" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
     </row>
     <row r="132" spans="1:8" ht="403.2">
@@ -26736,7 +27009,7 @@
         <v>327</v>
       </c>
       <c r="H132" s="3" t="s">
-        <v>765</v>
+        <v>762</v>
       </c>
     </row>
     <row r="133" spans="1:8">
@@ -26762,7 +27035,7 @@
         <v>330</v>
       </c>
       <c r="H133" s="6" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
     </row>
     <row r="134" spans="1:8" ht="43.2">
@@ -26788,7 +27061,7 @@
         <v>332</v>
       </c>
       <c r="H134" s="6" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
     </row>
     <row r="135" spans="1:8" ht="100.8">
@@ -26802,7 +27075,7 @@
         <v>2</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>761</v>
+        <v>758</v>
       </c>
       <c r="E135" s="2" t="s">
         <v>11</v>
@@ -26811,24 +27084,24 @@
         <v>12</v>
       </c>
       <c r="G135" s="3" t="s">
-        <v>762</v>
+        <v>759</v>
       </c>
       <c r="H135" s="3" t="s">
-        <v>740</v>
+        <v>737</v>
       </c>
     </row>
     <row r="136" spans="1:8" ht="115.2">
       <c r="A136" s="2" t="s">
-        <v>771</v>
+        <v>768</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>781</v>
+        <v>778</v>
       </c>
       <c r="C136" s="2">
         <v>0</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
       <c r="E136" s="2" t="s">
         <v>11</v>
@@ -26837,10 +27110,10 @@
         <v>12</v>
       </c>
       <c r="G136" s="3" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
       <c r="H136" s="3" t="s">
-        <v>784</v>
+        <v>781</v>
       </c>
     </row>
     <row r="137" spans="1:8" ht="409.6">
@@ -26866,7 +27139,7 @@
         <v>334</v>
       </c>
       <c r="H137" s="3" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
     </row>
     <row r="138" spans="1:8" ht="28.8">
@@ -26892,7 +27165,7 @@
         <v>337</v>
       </c>
       <c r="H138" s="6" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
     </row>
     <row r="139" spans="1:8">
@@ -26918,7 +27191,7 @@
         <v>340</v>
       </c>
       <c r="H139" s="6" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
     </row>
     <row r="140" spans="1:8" ht="57.6">
@@ -26944,7 +27217,7 @@
         <v>342</v>
       </c>
       <c r="H140" s="6" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
     </row>
     <row r="141" spans="1:8">
@@ -26970,7 +27243,7 @@
         <v>344</v>
       </c>
       <c r="H141" s="6" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
     </row>
     <row r="142" spans="1:8" ht="43.2">
@@ -26996,7 +27269,7 @@
         <v>346</v>
       </c>
       <c r="H142" s="6" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
     </row>
     <row r="143" spans="1:8" ht="86.4">
@@ -27022,7 +27295,7 @@
         <v>348</v>
       </c>
       <c r="H143" s="3" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
     </row>
     <row r="144" spans="1:8" ht="216">
@@ -27048,7 +27321,7 @@
         <v>350</v>
       </c>
       <c r="H144" s="3" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
     </row>
     <row r="145" spans="1:8" ht="86.4">
@@ -27100,7 +27373,7 @@
         <v>356</v>
       </c>
       <c r="H146" s="3" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
     </row>
     <row r="147" spans="1:8">
@@ -27152,7 +27425,7 @@
         <v>362</v>
       </c>
       <c r="H148" s="3" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
     </row>
     <row r="149" spans="1:8" ht="28.8">
@@ -27178,7 +27451,7 @@
         <v>365</v>
       </c>
       <c r="H149" s="3" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
     </row>
     <row r="150" spans="1:8">
@@ -27204,7 +27477,7 @@
         <v>367</v>
       </c>
       <c r="H150" s="3" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
     </row>
     <row r="151" spans="1:8" ht="129.6">
@@ -27230,7 +27503,7 @@
         <v>370</v>
       </c>
       <c r="H151" s="3" t="s">
-        <v>766</v>
+        <v>763</v>
       </c>
     </row>
     <row r="152" spans="1:8" ht="28.8">
@@ -27308,7 +27581,7 @@
         <v>379</v>
       </c>
       <c r="H154" s="3" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
     </row>
     <row r="155" spans="1:8" ht="28.8">
@@ -27334,7 +27607,7 @@
         <v>382</v>
       </c>
       <c r="H155" s="6" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="156" spans="1:8" ht="409.6">
@@ -27360,7 +27633,7 @@
         <v>384</v>
       </c>
       <c r="H156" s="3" t="s">
-        <v>741</v>
+        <v>738</v>
       </c>
     </row>
     <row r="157" spans="1:8" ht="43.2">
@@ -27386,7 +27659,7 @@
         <v>387</v>
       </c>
       <c r="H157" s="6" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
     </row>
     <row r="158" spans="1:8" ht="86.4">
@@ -27464,7 +27737,7 @@
         <v>396</v>
       </c>
       <c r="H160" s="6" t="s">
-        <v>742</v>
+        <v>739</v>
       </c>
     </row>
     <row r="161" spans="1:8" ht="100.8">
@@ -27490,7 +27763,7 @@
         <v>399</v>
       </c>
       <c r="H161" s="3" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="162" spans="1:8" ht="144">
@@ -27516,7 +27789,7 @@
         <v>401</v>
       </c>
       <c r="H162" s="3" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
     </row>
     <row r="163" spans="1:8" ht="100.8">
@@ -27542,7 +27815,7 @@
         <v>404</v>
       </c>
       <c r="H163" s="3" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
     </row>
     <row r="164" spans="1:8" ht="43.2">
@@ -27568,7 +27841,7 @@
         <v>406</v>
       </c>
       <c r="H164" s="6" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
     </row>
     <row r="165" spans="1:8" ht="115.2">
@@ -27594,7 +27867,7 @@
         <v>409</v>
       </c>
       <c r="H165" s="3" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
     </row>
     <row r="166" spans="1:8" ht="86.4">
@@ -27672,7 +27945,7 @@
         <v>419</v>
       </c>
       <c r="H168" s="3" t="s">
-        <v>744</v>
+        <v>741</v>
       </c>
     </row>
     <row r="169" spans="1:8" ht="57.6">
@@ -27724,7 +27997,7 @@
         <v>424</v>
       </c>
       <c r="H170" s="3" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
     </row>
     <row r="171" spans="1:8" ht="57.6">
@@ -27750,7 +28023,7 @@
         <v>427</v>
       </c>
       <c r="H171" s="6" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
     </row>
     <row r="172" spans="1:8" ht="28.8">
@@ -27825,10 +28098,10 @@
         <v>12</v>
       </c>
       <c r="G174" s="3" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="H174" s="3" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
     </row>
     <row r="175" spans="1:8" ht="28.8">
@@ -27877,10 +28150,10 @@
         <v>12</v>
       </c>
       <c r="G176" s="3" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="H176" s="3" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
     </row>
     <row r="177" spans="1:8" ht="201.6">
@@ -27906,7 +28179,7 @@
         <v>442</v>
       </c>
       <c r="H177" s="3" t="s">
-        <v>775</v>
+        <v>772</v>
       </c>
     </row>
     <row r="178" spans="1:8" ht="86.4">
@@ -27932,7 +28205,7 @@
         <v>445</v>
       </c>
       <c r="H178" s="3" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
     </row>
     <row r="179" spans="1:8">
@@ -27984,7 +28257,7 @@
         <v>451</v>
       </c>
       <c r="H180" s="6" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
     </row>
     <row r="181" spans="1:8">
@@ -28010,7 +28283,7 @@
         <v>454</v>
       </c>
       <c r="H181" s="6" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
     </row>
     <row r="182" spans="1:8">
@@ -28036,7 +28309,7 @@
         <v>457</v>
       </c>
       <c r="H182" s="6" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
     </row>
     <row r="183" spans="1:8">
@@ -28062,7 +28335,7 @@
         <v>460</v>
       </c>
       <c r="H183" s="6" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
     </row>
     <row r="184" spans="1:8">
@@ -28088,7 +28361,7 @@
         <v>463</v>
       </c>
       <c r="H184" s="6" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
     </row>
     <row r="185" spans="1:8" ht="144">
@@ -28114,7 +28387,7 @@
         <v>466</v>
       </c>
       <c r="H185" s="3" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
     </row>
     <row r="186" spans="1:8" ht="28.8">
@@ -28348,7 +28621,7 @@
         <v>492</v>
       </c>
       <c r="H194" s="6" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
     </row>
     <row r="195" spans="1:8">
@@ -28426,7 +28699,7 @@
         <v>500</v>
       </c>
       <c r="H197" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
     </row>
     <row r="198" spans="1:8">
@@ -28452,7 +28725,7 @@
         <v>502</v>
       </c>
       <c r="H198" s="6" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
     </row>
     <row r="199" spans="1:8" ht="100.8">
@@ -28478,7 +28751,7 @@
         <v>504</v>
       </c>
       <c r="H199" s="3" t="s">
-        <v>768</v>
+        <v>765</v>
       </c>
     </row>
     <row r="200" spans="1:8" ht="158.4">
@@ -28504,7 +28777,7 @@
         <v>506</v>
       </c>
       <c r="H200" s="3" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
     </row>
     <row r="201" spans="1:8" ht="43.2">
@@ -28530,7 +28803,7 @@
         <v>508</v>
       </c>
       <c r="H201" s="3" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
     </row>
     <row r="202" spans="1:8" ht="100.8">
@@ -28556,7 +28829,7 @@
         <v>510</v>
       </c>
       <c r="H202" s="3" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
     </row>
     <row r="203" spans="1:8" ht="43.2">
@@ -28582,7 +28855,7 @@
         <v>512</v>
       </c>
       <c r="H203" s="3" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
     </row>
     <row r="204" spans="1:8" ht="100.8">
@@ -28608,7 +28881,7 @@
         <v>514</v>
       </c>
       <c r="H204" s="3" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
     </row>
     <row r="205" spans="1:8" ht="100.8">
@@ -28634,7 +28907,7 @@
         <v>516</v>
       </c>
       <c r="H205" s="3" t="s">
-        <v>748</v>
+        <v>745</v>
       </c>
     </row>
     <row r="206" spans="1:8" ht="115.2">
@@ -28660,7 +28933,7 @@
         <v>518</v>
       </c>
       <c r="H206" s="3" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
     </row>
     <row r="207" spans="1:8" ht="158.4">
@@ -28686,7 +28959,7 @@
         <v>520</v>
       </c>
       <c r="H207" s="3" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
     </row>
     <row r="208" spans="1:8" ht="172.8">
@@ -28712,10 +28985,10 @@
         <v>522</v>
       </c>
       <c r="H208" s="3" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
     </row>
-    <row r="209" spans="1:8" ht="115.2">
+    <row r="209" spans="1:9" ht="115.2">
       <c r="A209" s="2" t="s">
         <v>8</v>
       </c>
@@ -28738,10 +29011,10 @@
         <v>524</v>
       </c>
       <c r="H209" s="3" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
     </row>
-    <row r="210" spans="1:8" ht="158.4">
+    <row r="210" spans="1:9" ht="158.4">
       <c r="A210" s="2" t="s">
         <v>8</v>
       </c>
@@ -28761,13 +29034,13 @@
         <v>12</v>
       </c>
       <c r="G210" s="3" t="s">
-        <v>769</v>
+        <v>766</v>
       </c>
       <c r="H210" s="3" t="s">
-        <v>770</v>
+        <v>767</v>
       </c>
     </row>
-    <row r="211" spans="1:8" ht="158.4">
+    <row r="211" spans="1:9" ht="158.4">
       <c r="A211" s="2" t="s">
         <v>8</v>
       </c>
@@ -28790,10 +29063,10 @@
         <v>527</v>
       </c>
       <c r="H211" s="3" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
     </row>
-    <row r="212" spans="1:8" ht="100.8">
+    <row r="212" spans="1:9" ht="100.8">
       <c r="A212" s="2" t="s">
         <v>8</v>
       </c>
@@ -28816,10 +29089,10 @@
         <v>529</v>
       </c>
       <c r="H212" s="3" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
     </row>
-    <row r="213" spans="1:8" ht="100.8">
+    <row r="213" spans="1:9" ht="100.8">
       <c r="A213" s="2" t="s">
         <v>8</v>
       </c>
@@ -28842,10 +29115,10 @@
         <v>531</v>
       </c>
       <c r="H213" s="3" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
     </row>
-    <row r="214" spans="1:8" ht="43.2">
+    <row r="214" spans="1:9" ht="43.2">
       <c r="A214" s="2" t="s">
         <v>8</v>
       </c>
@@ -28868,10 +29141,10 @@
         <v>533</v>
       </c>
       <c r="H214" s="3" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
     </row>
-    <row r="215" spans="1:8" ht="43.2">
+    <row r="215" spans="1:9" ht="43.2">
       <c r="A215" s="2" t="s">
         <v>8</v>
       </c>
@@ -28897,7 +29170,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="216" spans="1:8" ht="43.2">
+    <row r="216" spans="1:9" ht="43.2">
       <c r="A216" s="2" t="s">
         <v>8</v>
       </c>
@@ -28920,10 +29193,10 @@
         <v>538</v>
       </c>
       <c r="H216" s="3" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
     </row>
-    <row r="217" spans="1:8" ht="288">
+    <row r="217" spans="1:9" ht="409.6">
       <c r="A217" s="2" t="s">
         <v>8</v>
       </c>
@@ -28934,7 +29207,7 @@
         <v>21</v>
       </c>
       <c r="D217" s="2" t="s">
-        <v>539</v>
+        <v>795</v>
       </c>
       <c r="E217" s="2" t="s">
         <v>11</v>
@@ -28943,13 +29216,14 @@
         <v>12</v>
       </c>
       <c r="G217" s="3" t="s">
-        <v>540</v>
+        <v>796</v>
       </c>
       <c r="H217" s="3" t="s">
-        <v>723</v>
-      </c>
+        <v>797</v>
+      </c>
+      <c r="I217" s="3"/>
     </row>
-    <row r="218" spans="1:8" ht="115.2">
+    <row r="218" spans="1:9" ht="115.2">
       <c r="A218" s="2" t="s">
         <v>8</v>
       </c>
@@ -28960,7 +29234,7 @@
         <v>22</v>
       </c>
       <c r="D218" s="2" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="E218" s="2" t="s">
         <v>11</v>
@@ -28969,13 +29243,13 @@
         <v>12</v>
       </c>
       <c r="G218" s="3" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="H218" s="3" t="s">
-        <v>724</v>
+        <v>721</v>
       </c>
     </row>
-    <row r="219" spans="1:8" ht="43.2">
+    <row r="219" spans="1:9" ht="43.2">
       <c r="A219" s="2" t="s">
         <v>8</v>
       </c>
@@ -28986,7 +29260,7 @@
         <v>23</v>
       </c>
       <c r="D219" s="2" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="E219" s="2" t="s">
         <v>11</v>
@@ -28995,13 +29269,13 @@
         <v>12</v>
       </c>
       <c r="G219" s="3" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="H219" s="3" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
     </row>
-    <row r="220" spans="1:8" ht="86.4">
+    <row r="220" spans="1:9" ht="86.4">
       <c r="A220" s="2" t="s">
         <v>8</v>
       </c>
@@ -29012,7 +29286,7 @@
         <v>24</v>
       </c>
       <c r="D220" s="2" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="E220" s="2" t="s">
         <v>11</v>
@@ -29021,13 +29295,13 @@
         <v>12</v>
       </c>
       <c r="G220" s="3" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="H220" s="3" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
     </row>
-    <row r="221" spans="1:8" ht="115.2">
+    <row r="221" spans="1:9" ht="115.2">
       <c r="A221" s="2" t="s">
         <v>8</v>
       </c>
@@ -29038,7 +29312,7 @@
         <v>25</v>
       </c>
       <c r="D221" s="2" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="E221" s="2" t="s">
         <v>11</v>
@@ -29047,13 +29321,13 @@
         <v>12</v>
       </c>
       <c r="G221" s="3" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="H221" s="3" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
     </row>
-    <row r="222" spans="1:8" ht="43.2">
+    <row r="222" spans="1:9" ht="43.2">
       <c r="A222" s="2" t="s">
         <v>8</v>
       </c>
@@ -29064,7 +29338,7 @@
         <v>26</v>
       </c>
       <c r="D222" s="2" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="E222" s="2" t="s">
         <v>11</v>
@@ -29073,13 +29347,13 @@
         <v>12</v>
       </c>
       <c r="G222" s="3" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="H222" s="3" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
     </row>
-    <row r="223" spans="1:8" ht="100.8">
+    <row r="223" spans="1:9" ht="100.8">
       <c r="A223" s="2" t="s">
         <v>8</v>
       </c>
@@ -29090,7 +29364,7 @@
         <v>27</v>
       </c>
       <c r="D223" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="E223" s="2" t="s">
         <v>11</v>
@@ -29099,13 +29373,13 @@
         <v>12</v>
       </c>
       <c r="G223" s="3" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="H223" s="3" t="s">
-        <v>749</v>
+        <v>746</v>
       </c>
     </row>
-    <row r="224" spans="1:8" ht="43.2">
+    <row r="224" spans="1:9" ht="43.2">
       <c r="A224" s="2" t="s">
         <v>8</v>
       </c>
@@ -29116,7 +29390,7 @@
         <v>28</v>
       </c>
       <c r="D224" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="E224" s="2" t="s">
         <v>11</v>
@@ -29125,10 +29399,10 @@
         <v>12</v>
       </c>
       <c r="G224" s="3" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="H224" s="3" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="225" spans="1:8" ht="43.2">
@@ -29142,7 +29416,7 @@
         <v>29</v>
       </c>
       <c r="D225" s="2" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="E225" s="2" t="s">
         <v>11</v>
@@ -29151,10 +29425,10 @@
         <v>12</v>
       </c>
       <c r="G225" s="3" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="H225" s="3" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
     </row>
     <row r="226" spans="1:8" ht="100.8">
@@ -29168,7 +29442,7 @@
         <v>30</v>
       </c>
       <c r="D226" s="2" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="E226" s="2" t="s">
         <v>11</v>
@@ -29177,10 +29451,10 @@
         <v>12</v>
       </c>
       <c r="G226" s="3" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H226" s="3" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
     </row>
     <row r="227" spans="1:8" ht="28.8">
@@ -29188,13 +29462,13 @@
         <v>8</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="C227" s="2">
         <v>0</v>
       </c>
       <c r="D227" s="2" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="E227" s="2" t="s">
         <v>11</v>
@@ -29203,10 +29477,10 @@
         <v>12</v>
       </c>
       <c r="G227" s="3" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="H227" s="6" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
     </row>
     <row r="228" spans="1:8" ht="28.8">
@@ -29214,13 +29488,13 @@
         <v>8</v>
       </c>
       <c r="B228" s="2" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="C228" s="2">
         <v>0</v>
       </c>
       <c r="D228" s="2" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="E228" s="2" t="s">
         <v>11</v>
@@ -29229,10 +29503,10 @@
         <v>12</v>
       </c>
       <c r="G228" s="3" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="H228" s="3" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
     </row>
     <row r="229" spans="1:8" ht="43.2">
@@ -29240,13 +29514,13 @@
         <v>8</v>
       </c>
       <c r="B229" s="2" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="C229" s="2">
         <v>1</v>
       </c>
       <c r="D229" s="2" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="E229" s="2" t="s">
         <v>11</v>
@@ -29255,10 +29529,10 @@
         <v>12</v>
       </c>
       <c r="G229" s="3" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="H229" s="3" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
     </row>
     <row r="230" spans="1:8" ht="100.8">
@@ -29266,13 +29540,13 @@
         <v>8</v>
       </c>
       <c r="B230" s="2" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="C230" s="2">
         <v>2</v>
       </c>
       <c r="D230" s="2" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="E230" s="2" t="s">
         <v>11</v>
@@ -29281,10 +29555,10 @@
         <v>12</v>
       </c>
       <c r="G230" s="3" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="H230" s="3" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
     </row>
     <row r="231" spans="1:8" ht="43.2">
@@ -29292,13 +29566,13 @@
         <v>8</v>
       </c>
       <c r="B231" s="2" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="C231" s="2">
         <v>3</v>
       </c>
       <c r="D231" s="2" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="E231" s="2" t="s">
         <v>11</v>
@@ -29307,10 +29581,10 @@
         <v>12</v>
       </c>
       <c r="G231" s="3" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="H231" s="3" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
     </row>
     <row r="232" spans="1:8">
@@ -29318,13 +29592,13 @@
         <v>8</v>
       </c>
       <c r="B232" s="2" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="C232" s="2">
         <v>0</v>
       </c>
       <c r="D232" s="2" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="E232" s="2" t="s">
         <v>11</v>
@@ -29333,10 +29607,10 @@
         <v>12</v>
       </c>
       <c r="G232" s="3" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="H232" s="6" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
     </row>
     <row r="233" spans="1:8">
@@ -29344,13 +29618,13 @@
         <v>8</v>
       </c>
       <c r="B233" s="2" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="C233" s="2">
         <v>0</v>
       </c>
       <c r="D233" s="2" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="E233" s="2" t="s">
         <v>11</v>
@@ -29359,10 +29633,10 @@
         <v>12</v>
       </c>
       <c r="G233" s="3" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="H233" s="6" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
     </row>
     <row r="234" spans="1:8" ht="28.8">
@@ -29370,13 +29644,13 @@
         <v>8</v>
       </c>
       <c r="B234" s="2" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="C234" s="2">
         <v>1</v>
       </c>
       <c r="D234" s="2" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="E234" s="2" t="s">
         <v>11</v>
@@ -29385,10 +29659,10 @@
         <v>12</v>
       </c>
       <c r="G234" s="3" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="H234" s="6" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
     </row>
     <row r="235" spans="1:8">
@@ -29396,13 +29670,13 @@
         <v>8</v>
       </c>
       <c r="B235" s="2" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="C235" s="2">
         <v>0</v>
       </c>
       <c r="D235" s="2" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="E235" s="2" t="s">
         <v>11</v>
@@ -29411,10 +29685,10 @@
         <v>12</v>
       </c>
       <c r="G235" s="3" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="H235" s="6" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
     </row>
     <row r="236" spans="1:8" ht="28.8">
@@ -29422,13 +29696,13 @@
         <v>8</v>
       </c>
       <c r="B236" s="2" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="C236" s="2">
         <v>1</v>
       </c>
       <c r="D236" s="2" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="E236" s="2" t="s">
         <v>11</v>
@@ -29437,10 +29711,10 @@
         <v>12</v>
       </c>
       <c r="G236" s="3" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="H236" s="4" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
     </row>
     <row r="237" spans="1:8">
@@ -29448,13 +29722,13 @@
         <v>8</v>
       </c>
       <c r="B237" s="2" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="C237" s="2">
         <v>0</v>
       </c>
       <c r="D237" s="2" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="E237" s="2" t="s">
         <v>11</v>
@@ -29463,7 +29737,7 @@
         <v>12</v>
       </c>
       <c r="G237" s="3" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="H237" s="4" t="s">
         <v>25</v>
@@ -29474,13 +29748,13 @@
         <v>8</v>
       </c>
       <c r="B238" s="2" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="C238" s="2">
         <v>1</v>
       </c>
       <c r="D238" s="2" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="E238" s="2" t="s">
         <v>11</v>
@@ -29489,10 +29763,10 @@
         <v>12</v>
       </c>
       <c r="G238" s="3" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="H238" s="4" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
     </row>
     <row r="239" spans="1:8">
@@ -29500,13 +29774,13 @@
         <v>8</v>
       </c>
       <c r="B239" s="2" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="C239" s="2">
         <v>0</v>
       </c>
       <c r="D239" s="2" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="E239" s="2" t="s">
         <v>11</v>
@@ -29515,24 +29789,24 @@
         <v>12</v>
       </c>
       <c r="G239" s="3" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="H239" s="4" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
     </row>
     <row r="240" spans="1:8">
       <c r="A240" t="s">
-        <v>771</v>
+        <v>768</v>
       </c>
       <c r="B240" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="C240">
         <v>1</v>
       </c>
       <c r="D240" t="s">
-        <v>772</v>
+        <v>769</v>
       </c>
       <c r="E240" t="s">
         <v>11</v>
@@ -29541,10 +29815,10 @@
         <v>12</v>
       </c>
       <c r="G240" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="H240" s="4" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
     </row>
     <row r="241" spans="1:8">

</xml_diff>

<commit_message>
removed id: welcome inline language picker while waiting on fix
</commit_message>
<xml_diff>
--- a/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
+++ b/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6216AE60-B8D2-4472-A453-4D0A62E5BC07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{270D9FCB-92ED-4F26-8FEB-ACFC17602995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-31905" yWindow="-3210" windowWidth="26445" windowHeight="16770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-34950" yWindow="3765" windowWidth="26445" windowHeight="16770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22162,243 +22162,6 @@
     </r>
   </si>
   <si>
-    <t>31a3791a34401744a473ea590edf5be1</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ get_language_list(lang_codes=al_interview_languages, current=al_user_language) }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Welcome to Illinois Legal Aid Online's **Power of Attorney for Health Care** Easy Form.
-This program helps you make documents that give someone you trust power of attorney to make decisions about your health care. This means they can make choices about your health care when you cannot. You can also let them make choices about your health care earlier, if you choose.
-This program has videos with information about making a Power of Attorney for Health Care. You do not have to watch them, but you may find them helpful.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if user_path == "Shirley":
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[YOUTUBE 7qy101TRdiI]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% elif user_path == "Frederico" or user_path == "Federico":
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[YOUTUBE GR9t6ygX13g]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% elif user_path == "Lisa":
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[YOUTUBE h2ZGl568xHo]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-To learn more, read ILAO's article about [**Power of Attorney for Health Care basics**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://www.illinoislegalaid.org/legal-information/setting-power-attorney-healthcare</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">).
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">${ get_language_list(lang_codes=al_interview_languages, current=al_user_language) }
-Bienvenido(a) al Formulario Guiado de Poder Notarial para el Cuidado de la Salud de Illinois Legal Aid Online.
-Este programa te ayuda a crear documentos que le otorgan a una persona de tu confianza la autoridad legal para tomar decisiones sobre tu atención médica. Esto significa que esa persona podrá tomar decisiones sobre tu atención médica cuando no puedas hacerlo por ti mismo(a). Si así lo deseas, también puedes autorizarla para que tome decisiones sobre tu atención médica antesde que eso ocurra.
-Este programa incluye videos con información sobre cómo hacer un Poder Notarial para el Cuidado de la Salud. No tienes que verlos, pero pueden serte útiles.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">[YOUTUBE ccToVpEse7s]
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Para obtener más información, lee el artículo de ILAO sobre los [**Conceptos Básicos del Poder Notarial para el Cuidado de la Salud**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org/legal-information/setting-power-attorney-healthcare</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>).</t>
-    </r>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">**Límites para </t>
     </r>
@@ -23177,6 +22940,250 @@
       <t xml:space="preserve">
 **Nota:** El Poder Notarial debe firmarse frente a al menos un testigo para que sea válido.
 ¡Gracias por usar los Formularios Guiados de ILAO!</t>
+    </r>
+  </si>
+  <si>
+    <t>80b04da1b3097b769fbc55dc4f8a6d71</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Welcome to Illinois Legal Aid Online's **Power of Attorney for Health Care** Easy Form.
+This program helps you make documents that give someone you trust power of attorney to make decisions about your health care. This means they can make choices about your health care when you cannot. You can also let them make choices about your health care earlier, if you choose.
+This program has videos with information about making a Power of Attorney for Health Care. You do not have to watch them, but you may find them helpful.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if user_path == "Shirley":
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[YOUTUBE 7qy101TRdiI]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% elif user_path == "Frederico" or user_path == "Federico":
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[YOUTUBE GR9t6ygX13g]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% elif user_path == "Lisa":
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[YOUTUBE h2ZGl568xHo]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+To learn more, read ILAO's article about </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[**Power of Attorney for Health Care basics**]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://www.illinoislegalaid.org/legal-information/setting-power-attorney-healthcare</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">).
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Bienvenido(a) al Formulario Guiado de Poder Notarial para el Cuidado de la Salud de Illinois Legal Aid Online.
+Este programa te ayuda a crear documentos que le otorgan a una persona de tu confianza la autoridad legal para tomar decisiones sobre tu atención médica. Esto significa que esa persona podrá tomar decisiones sobre tu atención médica cuando no puedas hacerlo por ti mismo(a). Si así lo deseas, también puedes autorizarla para que tome decisiones sobre tu atención médica antesde que eso ocurra.
+Este programa incluye videos con información sobre cómo hacer un Poder Notarial para el Cuidado de la Salud. No tienes que verlos, pero pueden serte útiles.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">[YOUTUBE ccToVpEse7s]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Para obtener más información, lee el artículo de ILAO sobre los [**Conceptos Básicos del Poder Notarial para el Cuidado de la Salud**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/legal-information/setting-power-attorney-healthcare</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).</t>
     </r>
   </si>
 </sst>
@@ -23705,7 +23712,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="345.6">
+    <row r="3" spans="1:8" ht="316.8">
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
@@ -23716,7 +23723,7 @@
         <v>1</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>11</v>
@@ -23725,10 +23732,10 @@
         <v>12</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>792</v>
+        <v>796</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>793</v>
+        <v>797</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -28214,7 +28221,7 @@
         <v>1</v>
       </c>
       <c r="D176" s="2" t="s">
-        <v>795</v>
+        <v>792</v>
       </c>
       <c r="E176" s="2" t="s">
         <v>11</v>
@@ -28223,10 +28230,10 @@
         <v>12</v>
       </c>
       <c r="G176" s="3" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
       <c r="H176" s="3" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
     </row>
     <row r="177" spans="1:8" ht="201.6">
@@ -29292,7 +29299,7 @@
         <v>790</v>
       </c>
       <c r="H217" s="3" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
       <c r="I217" s="3"/>
     </row>

</xml_diff>

<commit_message>
adjusted language selection options
</commit_message>
<xml_diff>
--- a/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
+++ b/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{270D9FCB-92ED-4F26-8FEB-ACFC17602995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81486406-1880-4DF9-B9C7-20B763325E4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-34950" yWindow="3765" windowWidth="26445" windowHeight="16770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1164" yWindow="936" windowWidth="21156" windowHeight="13416" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22943,18 +22943,30 @@
     </r>
   </si>
   <si>
-    <t>80b04da1b3097b769fbc55dc4f8a6d71</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Welcome to Illinois Legal Aid Online's **Power of Attorney for Health Care** Easy Form.
+    <t>7ae3790d22f601b38af6ba8ae684093e</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ get_language_list(lang_codes=al_interview_languages, current=get_language()) }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Welcome to Illinois Legal Aid Online's **Power of Attorney for Health Care** Easy Form.
 This program helps you make documents that give someone you trust power of attorney to make decisions about your health care. This means they can make choices about your health care when you cannot. You can also let them make choices about your health care earlier, if you choose.
 This program has videos with information about making a Power of Attorney for Health Care. You do not have to watch them, but you may find them helpful.
 </t>
@@ -23136,7 +23148,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">Bienvenido(a) al Formulario Guiado de Poder Notarial para el Cuidado de la Salud de Illinois Legal Aid Online.
+      <t xml:space="preserve">${ get_language_list(lang_codes=al_interview_languages, current=get_language()) }
+Bienvenido(a) al Formulario Guiado de Poder Notarial para el Cuidado de la Salud de Illinois Legal Aid Online.
 Este programa te ayuda a crear documentos que le otorgan a una persona de tu confianza la autoridad legal para tomar decisiones sobre tu atención médica. Esto significa que esa persona podrá tomar decisiones sobre tu atención médica cuando no puedas hacerlo por ti mismo(a). Si así lo deseas, también puedes autorizarla para que tome decisiones sobre tu atención médica antesde que eso ocurra.
 Este programa incluye videos con información sobre cómo hacer un Poder Notarial para el Cuidado de la Salud. No tienes que verlos, pero pueden serte útiles.
 </t>
@@ -23712,7 +23725,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="316.8">
+    <row r="3" spans="1:8" ht="345.6">
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
review screen tweak adjust es filenames remove inline lang picker
</commit_message>
<xml_diff>
--- a/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
+++ b/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81486406-1880-4DF9-B9C7-20B763325E4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AD69830-080F-4232-A12C-AFFA3E5058E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1164" yWindow="936" windowWidth="21156" windowHeight="13416" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-35400" yWindow="-3195" windowWidth="30840" windowHeight="16845" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -16491,211 +16491,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">**Instrucciones sobre la disposición de tus restos:** 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if self_remains_preference != "specific":
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${self_remains_preference}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${self_specific_burial_preference}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>% endif</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">**Instrucciones sobre la disposición de los restos de </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${principal.name_full()}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">**:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if other_remains_preference != "specific":
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${other_remains_preference}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${other_specific_burial_preference}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>% endif</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
       <t xml:space="preserve">**¿Quisieras donar tus órganos?**  
 </t>
     </r>
@@ -22943,30 +22738,77 @@
     </r>
   </si>
   <si>
-    <t>7ae3790d22f601b38af6ba8ae684093e</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ get_language_list(lang_codes=al_interview_languages, current=get_language()) }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Bienvenido(a) al Formulario Guiado de Poder Notarial para el Cuidado de la Salud de Illinois Legal Aid Online.
+Este programa te ayuda a crear documentos que le otorgan a una persona de tu confianza la autoridad legal para tomar decisiones sobre tu atención médica. Esto significa que esa persona podrá tomar decisiones sobre tu atención médica cuando no puedas hacerlo por ti mismo(a). Si así lo deseas, también puedes autorizarla para que tome decisiones sobre tu atención médica antesde que eso ocurra.
+Este programa incluye videos con información sobre cómo hacer un Poder Notarial para el Cuidado de la Salud. No tienes que verlos, pero pueden serte útiles.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">[YOUTUBE ccToVpEse7s]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-Welcome to Illinois Legal Aid Online's **Power of Attorney for Health Care** Easy Form.
+Para obtener más información, lee el artículo de ILAO sobre los [**Conceptos Básicos del Poder Notarial para el Cuidado de la Salud**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/legal-information/setting-power-attorney-healthcare</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).</t>
+    </r>
+  </si>
+  <si>
+    <t>80b04da1b3097b769fbc55dc4f8a6d71</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Welcome to Illinois Legal Aid Online's **Power of Attorney for Health Care** Easy Form.
 This program helps you make documents that give someone you trust power of attorney to make decisions about your health care. This means they can make choices about your health care when you cannot. You can also let them make choices about your health care earlier, if you choose.
 This program has videos with information about making a Power of Attorney for Health Care. You do not have to watch them, but you may find them helpful.
 </t>
@@ -23148,23 +22990,31 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">${ get_language_list(lang_codes=al_interview_languages, current=get_language()) }
-Bienvenido(a) al Formulario Guiado de Poder Notarial para el Cuidado de la Salud de Illinois Legal Aid Online.
-Este programa te ayuda a crear documentos que le otorgan a una persona de tu confianza la autoridad legal para tomar decisiones sobre tu atención médica. Esto significa que esa persona podrá tomar decisiones sobre tu atención médica cuando no puedas hacerlo por ti mismo(a). Si así lo deseas, también puedes autorizarla para que tome decisiones sobre tu atención médica antesde que eso ocurra.
-Este programa incluye videos con información sobre cómo hacer un Poder Notarial para el Cuidado de la Salud. No tienes que verlos, pero pueden serte útiles.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">[YOUTUBE ccToVpEse7s]
-</t>
+      <t xml:space="preserve">**Instrucciones sobre la disposición de tus restos: (En inglés)** 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if self_remains_preference != "specific":
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${self_remains_preference}</t>
     </r>
     <r>
       <rPr>
@@ -23175,28 +23025,165 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-Para obtener más información, lee el artículo de ILAO sobre los [**Conceptos Básicos del Poder Notarial para el Cuidado de la Salud**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org/legal-information/setting-power-attorney-healthcare</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>).</t>
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% else:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${self_specific_burial_preference}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>% endif</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">**Instrucciones sobre la disposición de los restos de </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${principal.name_full()} (En inglés)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">**:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if other_remains_preference != "specific":
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${other_remains_preference}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% else:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${other_specific_burial_preference}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>% endif</t>
     </r>
   </si>
 </sst>
@@ -23323,7 +23310,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -23348,6 +23335,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -23725,30 +23718,30 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="345.6">
+    <row r="3" spans="1:8" ht="316.8">
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="10">
         <v>1</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="10" t="s">
+        <v>794</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="11" t="s">
         <v>795</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>796</v>
-      </c>
       <c r="H3" s="7" t="s">
-        <v>797</v>
+        <v>793</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -23904,7 +23897,7 @@
         <v>31</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="28.8">
@@ -23918,7 +23911,7 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>11</v>
@@ -23927,7 +23920,7 @@
         <v>12</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>33</v>
@@ -23944,7 +23937,7 @@
         <v>1</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>11</v>
@@ -23953,7 +23946,7 @@
         <v>12</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>34</v>
@@ -24008,7 +24001,7 @@
         <v>40</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="28.8">
@@ -24060,7 +24053,7 @@
         <v>46</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="28.8">
@@ -24112,21 +24105,21 @@
         <v>52</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="115.2">
       <c r="A18" s="2" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="C18" s="2">
         <v>0</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>11</v>
@@ -24135,18 +24128,18 @@
         <v>12</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="28.8">
       <c r="A19" s="2" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="C19" s="2">
         <v>1</v>
@@ -24242,7 +24235,7 @@
         <v>63</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="57.6">
@@ -24268,7 +24261,7 @@
         <v>65</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="28.8">
@@ -24412,7 +24405,7 @@
         <v>1</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>11</v>
@@ -24421,10 +24414,10 @@
         <v>12</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -24528,7 +24521,7 @@
         <v>85</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -24866,7 +24859,7 @@
         <v>120</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -24996,7 +24989,7 @@
         <v>131</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="28.8">
@@ -25022,7 +25015,7 @@
         <v>133</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="28.8">
@@ -25100,7 +25093,7 @@
         <v>142</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
     </row>
     <row r="56" spans="1:8" ht="288">
@@ -25126,7 +25119,7 @@
         <v>144</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="28.8">
@@ -25464,7 +25457,7 @@
         <v>177</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
     </row>
     <row r="70" spans="1:8" ht="28.8">
@@ -25490,7 +25483,7 @@
         <v>179</v>
       </c>
       <c r="H70" s="9" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
     </row>
     <row r="71" spans="1:8">
@@ -25568,7 +25561,7 @@
         <v>185</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -25646,7 +25639,7 @@
         <v>193</v>
       </c>
       <c r="H76" s="3" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
     </row>
     <row r="77" spans="1:8" ht="115.2">
@@ -25698,7 +25691,7 @@
         <v>198</v>
       </c>
       <c r="H78" s="3" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
     </row>
     <row r="79" spans="1:8" ht="28.8">
@@ -25747,7 +25740,7 @@
         <v>12</v>
       </c>
       <c r="G80" s="3" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
       <c r="H80" s="3" t="s">
         <v>634</v>
@@ -25802,7 +25795,7 @@
         <v>207</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
     </row>
     <row r="83" spans="1:8">
@@ -25932,7 +25925,7 @@
         <v>220</v>
       </c>
       <c r="H87" s="6" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
     </row>
     <row r="88" spans="1:8" ht="43.2">
@@ -25984,7 +25977,7 @@
         <v>639</v>
       </c>
       <c r="H89" s="3" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
     </row>
     <row r="90" spans="1:8" ht="72">
@@ -26036,7 +26029,7 @@
         <v>228</v>
       </c>
       <c r="H91" s="3" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
     </row>
     <row r="92" spans="1:8">
@@ -26192,7 +26185,7 @@
         <v>243</v>
       </c>
       <c r="H97" s="6" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
     </row>
     <row r="98" spans="1:8" ht="129.6">
@@ -26218,7 +26211,7 @@
         <v>245</v>
       </c>
       <c r="H98" s="3" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
     </row>
     <row r="99" spans="1:8" ht="86.4">
@@ -26270,7 +26263,7 @@
         <v>250</v>
       </c>
       <c r="H100" s="3" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
     </row>
     <row r="101" spans="1:8" ht="28.8">
@@ -26553,7 +26546,7 @@
         <v>12</v>
       </c>
       <c r="G111" s="8" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
       <c r="H111" s="3" t="s">
         <v>651</v>
@@ -26894,7 +26887,7 @@
         <v>307</v>
       </c>
       <c r="H124" s="8" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
     </row>
     <row r="125" spans="1:8" ht="28.8">
@@ -26920,7 +26913,7 @@
         <v>309</v>
       </c>
       <c r="H125" s="8" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
     </row>
     <row r="126" spans="1:8" ht="28.8">
@@ -26946,7 +26939,7 @@
         <v>311</v>
       </c>
       <c r="H126" s="8" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
     </row>
     <row r="127" spans="1:8">
@@ -27024,7 +27017,7 @@
         <v>318</v>
       </c>
       <c r="H129" s="3" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
     </row>
     <row r="130" spans="1:8">
@@ -27102,7 +27095,7 @@
         <v>325</v>
       </c>
       <c r="H132" s="3" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
     </row>
     <row r="133" spans="1:8">
@@ -27168,7 +27161,7 @@
         <v>2</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="E135" s="2" t="s">
         <v>11</v>
@@ -27177,24 +27170,24 @@
         <v>12</v>
       </c>
       <c r="G135" s="3" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="H135" s="3" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
     </row>
     <row r="136" spans="1:8" ht="115.2">
       <c r="A136" s="2" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="C136" s="2">
         <v>0</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="E136" s="2" t="s">
         <v>11</v>
@@ -27203,10 +27196,10 @@
         <v>12</v>
       </c>
       <c r="G136" s="3" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="H136" s="3" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
     </row>
     <row r="137" spans="1:8" ht="409.6">
@@ -27232,7 +27225,7 @@
         <v>332</v>
       </c>
       <c r="H137" s="3" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
     </row>
     <row r="138" spans="1:8" ht="28.8">
@@ -27466,7 +27459,7 @@
         <v>354</v>
       </c>
       <c r="H146" s="3" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
     </row>
     <row r="147" spans="1:8">
@@ -27596,7 +27589,7 @@
         <v>368</v>
       </c>
       <c r="H151" s="3" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
     </row>
     <row r="152" spans="1:8" ht="28.8">
@@ -27726,7 +27719,7 @@
         <v>382</v>
       </c>
       <c r="H156" s="3" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
     </row>
     <row r="157" spans="1:8" ht="43.2">
@@ -27830,7 +27823,7 @@
         <v>394</v>
       </c>
       <c r="H160" s="6" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
     </row>
     <row r="161" spans="1:8" ht="100.8">
@@ -27882,7 +27875,7 @@
         <v>399</v>
       </c>
       <c r="H162" s="3" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
     </row>
     <row r="163" spans="1:8" ht="100.8">
@@ -28038,7 +28031,7 @@
         <v>417</v>
       </c>
       <c r="H168" s="3" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
     </row>
     <row r="169" spans="1:8" ht="57.6">
@@ -28194,7 +28187,7 @@
         <v>696</v>
       </c>
       <c r="H174" s="3" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
     </row>
     <row r="175" spans="1:8" ht="28.8">
@@ -28234,7 +28227,7 @@
         <v>1</v>
       </c>
       <c r="D176" s="2" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="E176" s="2" t="s">
         <v>11</v>
@@ -28243,10 +28236,10 @@
         <v>12</v>
       </c>
       <c r="G176" s="3" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="H176" s="3" t="s">
-        <v>794</v>
+        <v>792</v>
       </c>
     </row>
     <row r="177" spans="1:8" ht="201.6">
@@ -28272,7 +28265,7 @@
         <v>439</v>
       </c>
       <c r="H177" s="3" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
     </row>
     <row r="178" spans="1:8" ht="86.4">
@@ -28298,7 +28291,7 @@
         <v>442</v>
       </c>
       <c r="H178" s="3" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
     </row>
     <row r="179" spans="1:8">
@@ -28792,7 +28785,7 @@
         <v>497</v>
       </c>
       <c r="H197" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
     </row>
     <row r="198" spans="1:8">
@@ -28818,7 +28811,7 @@
         <v>499</v>
       </c>
       <c r="H198" s="6" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
     </row>
     <row r="199" spans="1:8" ht="100.8">
@@ -28844,7 +28837,7 @@
         <v>501</v>
       </c>
       <c r="H199" s="3" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
     </row>
     <row r="200" spans="1:8" ht="158.4">
@@ -29000,7 +28993,7 @@
         <v>513</v>
       </c>
       <c r="H205" s="3" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
     </row>
     <row r="206" spans="1:8" ht="115.2">
@@ -29127,10 +29120,10 @@
         <v>12</v>
       </c>
       <c r="G210" s="3" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="H210" s="3" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
     </row>
     <row r="211" spans="1:9" ht="158.4">
@@ -29182,7 +29175,7 @@
         <v>526</v>
       </c>
       <c r="H212" s="3" t="s">
-        <v>714</v>
+        <v>796</v>
       </c>
     </row>
     <row r="213" spans="1:9" ht="100.8">
@@ -29208,7 +29201,7 @@
         <v>528</v>
       </c>
       <c r="H213" s="3" t="s">
-        <v>715</v>
+        <v>797</v>
       </c>
     </row>
     <row r="214" spans="1:9" ht="43.2">
@@ -29234,7 +29227,7 @@
         <v>530</v>
       </c>
       <c r="H214" s="3" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
     </row>
     <row r="215" spans="1:9" ht="43.2">
@@ -29286,7 +29279,7 @@
         <v>535</v>
       </c>
       <c r="H216" s="3" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
     </row>
     <row r="217" spans="1:9" ht="409.6">
@@ -29300,7 +29293,7 @@
         <v>21</v>
       </c>
       <c r="D217" s="2" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="E217" s="2" t="s">
         <v>11</v>
@@ -29309,10 +29302,10 @@
         <v>12</v>
       </c>
       <c r="G217" s="3" t="s">
-        <v>790</v>
+        <v>788</v>
       </c>
       <c r="H217" s="3" t="s">
-        <v>791</v>
+        <v>789</v>
       </c>
       <c r="I217" s="3"/>
     </row>
@@ -29339,7 +29332,7 @@
         <v>537</v>
       </c>
       <c r="H218" s="3" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
     </row>
     <row r="219" spans="1:9" ht="43.2">
@@ -29469,7 +29462,7 @@
         <v>548</v>
       </c>
       <c r="H223" s="3" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
     </row>
     <row r="224" spans="1:9" ht="43.2">
@@ -29890,7 +29883,7 @@
     </row>
     <row r="240" spans="1:8">
       <c r="A240" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="B240" t="s">
         <v>590</v>
@@ -29899,7 +29892,7 @@
         <v>1</v>
       </c>
       <c r="D240" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="E240" t="s">
         <v>11</v>
@@ -29908,10 +29901,10 @@
         <v>12</v>
       </c>
       <c r="G240" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="H240" s="4" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
     </row>
     <row r="241" spans="1:8">

</xml_diff>

<commit_message>
update legal capacity definition
</commit_message>
<xml_diff>
--- a/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
+++ b/docassemble/PowerOfAttorneyHealthCare/data/sources/poa_hc_es.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AD69830-080F-4232-A12C-AFFA3E5058E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{726B4E2B-DC62-4DF1-8113-8FB901BCE7A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-35400" yWindow="-3195" windowWidth="30840" windowHeight="16845" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-36045" yWindow="-3345" windowWidth="30840" windowHeight="16845" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -5111,13 +5111,6 @@
     <t>legal capacity</t>
   </si>
   <si>
-    <t>eae54beffdc63e0f44821e6670d5495b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">You have the **legal capacity** to revoke a Power of Attorney for Health Care if you understand what you are signing and what it means for your future.
-</t>
-  </si>
-  <si>
     <t>58ca2de59caab479fb537acf8b4b6f5c</t>
   </si>
   <si>
@@ -13622,9 +13615,6 @@
     <t>Capacidad legal</t>
   </si>
   <si>
-    <t>Tienes capacidad legal para revocar un Poder Notarial para el Cuidado de la Salud si entiendes lo que estás firmando y lo que significa para tu futuro.</t>
-  </si>
-  <si>
     <t>**Video: ¿Qué es este periodo de reflexión de 30 días?**</t>
   </si>
   <si>
@@ -23185,6 +23175,16 @@
       </rPr>
       <t>% endif</t>
     </r>
+  </si>
+  <si>
+    <t>La **capacidad legal** significa que una persona puede entender lo que está firmando y lo que esto implica para su futuro.</t>
+  </si>
+  <si>
+    <t>758dbe9f10315dbb11909fb009a7a357</t>
+  </si>
+  <si>
+    <t xml:space="preserve">**Legal capacity** means a person is mentally able to understand what they are signing and understand what it means for their future.
+</t>
   </si>
 </sst>
 </file>
@@ -23725,23 +23725,23 @@
       <c r="B3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="2">
         <v>1</v>
       </c>
-      <c r="D3" s="10" t="s">
-        <v>794</v>
-      </c>
-      <c r="E3" s="10" t="s">
+      <c r="D3" s="2" t="s">
+        <v>791</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="11" t="s">
-        <v>795</v>
+      <c r="G3" s="3" t="s">
+        <v>792</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -23793,7 +23793,7 @@
         <v>20</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -23897,7 +23897,7 @@
         <v>31</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>744</v>
+        <v>741</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="28.8">
@@ -23911,7 +23911,7 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>749</v>
+        <v>746</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>11</v>
@@ -23920,7 +23920,7 @@
         <v>12</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>752</v>
+        <v>749</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>33</v>
@@ -23937,7 +23937,7 @@
         <v>1</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>750</v>
+        <v>747</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>11</v>
@@ -23946,7 +23946,7 @@
         <v>12</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>751</v>
+        <v>748</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>34</v>
@@ -24001,7 +24001,7 @@
         <v>40</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="28.8">
@@ -24053,7 +24053,7 @@
         <v>46</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>768</v>
+        <v>765</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="28.8">
@@ -24105,21 +24105,21 @@
         <v>52</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="115.2">
       <c r="A18" s="2" t="s">
-        <v>763</v>
+        <v>760</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>769</v>
+        <v>766</v>
       </c>
       <c r="C18" s="2">
         <v>0</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>770</v>
+        <v>767</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>11</v>
@@ -24128,18 +24128,18 @@
         <v>12</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>771</v>
+        <v>768</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>772</v>
+        <v>769</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="28.8">
       <c r="A19" s="2" t="s">
-        <v>763</v>
+        <v>760</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>769</v>
+        <v>766</v>
       </c>
       <c r="C19" s="2">
         <v>1</v>
@@ -24183,7 +24183,7 @@
         <v>58</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -24209,7 +24209,7 @@
         <v>61</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="43.2">
@@ -24235,7 +24235,7 @@
         <v>63</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="57.6">
@@ -24261,7 +24261,7 @@
         <v>65</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="28.8">
@@ -24287,7 +24287,7 @@
         <v>67</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="57.6">
@@ -24313,7 +24313,7 @@
         <v>69</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="28.8">
@@ -24339,7 +24339,7 @@
         <v>72</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="244.8">
@@ -24365,7 +24365,7 @@
         <v>74</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="86.4">
@@ -24391,7 +24391,7 @@
         <v>77</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="409.6">
@@ -24405,7 +24405,7 @@
         <v>1</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>11</v>
@@ -24414,10 +24414,10 @@
         <v>12</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>781</v>
+        <v>778</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -24443,7 +24443,7 @@
         <v>79</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -24469,7 +24469,7 @@
         <v>81</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -24495,7 +24495,7 @@
         <v>83</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -24521,7 +24521,7 @@
         <v>85</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>777</v>
+        <v>774</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -24573,7 +24573,7 @@
         <v>90</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="100.8">
@@ -24599,7 +24599,7 @@
         <v>93</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="28.8">
@@ -24625,7 +24625,7 @@
         <v>95</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="86.4">
@@ -24651,7 +24651,7 @@
         <v>98</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="28.8">
@@ -24677,7 +24677,7 @@
         <v>101</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="144">
@@ -24703,7 +24703,7 @@
         <v>103</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="86.4">
@@ -24755,7 +24755,7 @@
         <v>110</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="374.4">
@@ -24781,7 +24781,7 @@
         <v>112</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="86.4">
@@ -24807,7 +24807,7 @@
         <v>115</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="28.8">
@@ -24833,7 +24833,7 @@
         <v>117</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="28.8">
@@ -24859,7 +24859,7 @@
         <v>120</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -24885,7 +24885,7 @@
         <v>122</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="43.2">
@@ -24911,7 +24911,7 @@
         <v>124</v>
       </c>
       <c r="H48" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -24937,7 +24937,7 @@
         <v>126</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -24963,7 +24963,7 @@
         <v>128</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="129.6">
@@ -24989,7 +24989,7 @@
         <v>131</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="28.8">
@@ -25015,7 +25015,7 @@
         <v>133</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="28.8">
@@ -25067,7 +25067,7 @@
         <v>139</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
     </row>
     <row r="55" spans="1:8" ht="100.8">
@@ -25093,7 +25093,7 @@
         <v>142</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
     </row>
     <row r="56" spans="1:8" ht="288">
@@ -25119,7 +25119,7 @@
         <v>144</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="28.8">
@@ -25145,7 +25145,7 @@
         <v>147</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -25197,7 +25197,7 @@
         <v>153</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
     </row>
     <row r="60" spans="1:8" ht="28.8">
@@ -25223,7 +25223,7 @@
         <v>155</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
     </row>
     <row r="61" spans="1:8" ht="144">
@@ -25249,7 +25249,7 @@
         <v>157</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -25327,7 +25327,7 @@
         <v>165</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
     </row>
     <row r="65" spans="1:8" ht="43.2">
@@ -25353,7 +25353,7 @@
         <v>167</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="57.6">
@@ -25379,7 +25379,7 @@
         <v>169</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
     </row>
     <row r="67" spans="1:8">
@@ -25431,7 +25431,7 @@
         <v>175</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
     </row>
     <row r="69" spans="1:8" ht="172.8">
@@ -25457,7 +25457,7 @@
         <v>177</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>719</v>
+        <v>716</v>
       </c>
     </row>
     <row r="70" spans="1:8" ht="28.8">
@@ -25483,7 +25483,7 @@
         <v>179</v>
       </c>
       <c r="H70" s="9" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
     </row>
     <row r="71" spans="1:8">
@@ -25509,7 +25509,7 @@
         <v>181</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
     </row>
     <row r="72" spans="1:8" ht="43.2">
@@ -25535,7 +25535,7 @@
         <v>183</v>
       </c>
       <c r="H72" s="3" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
     </row>
     <row r="73" spans="1:8" ht="57.6">
@@ -25561,7 +25561,7 @@
         <v>185</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>722</v>
+        <v>719</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -25587,7 +25587,7 @@
         <v>187</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="28.8">
@@ -25639,7 +25639,7 @@
         <v>193</v>
       </c>
       <c r="H76" s="3" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
     </row>
     <row r="77" spans="1:8" ht="115.2">
@@ -25665,7 +25665,7 @@
         <v>196</v>
       </c>
       <c r="H77" s="3" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
     </row>
     <row r="78" spans="1:8" ht="360">
@@ -25691,7 +25691,7 @@
         <v>198</v>
       </c>
       <c r="H78" s="3" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
     </row>
     <row r="79" spans="1:8" ht="28.8">
@@ -25717,7 +25717,7 @@
         <v>201</v>
       </c>
       <c r="H79" s="6" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
     </row>
     <row r="80" spans="1:8" ht="28.8">
@@ -25740,10 +25740,10 @@
         <v>12</v>
       </c>
       <c r="G80" s="3" t="s">
-        <v>778</v>
+        <v>775</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
     </row>
     <row r="81" spans="1:8" ht="72">
@@ -25769,7 +25769,7 @@
         <v>205</v>
       </c>
       <c r="H81" s="3" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
     </row>
     <row r="82" spans="1:8" ht="72">
@@ -25795,7 +25795,7 @@
         <v>207</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>724</v>
+        <v>721</v>
       </c>
     </row>
     <row r="83" spans="1:8">
@@ -25847,7 +25847,7 @@
         <v>212</v>
       </c>
       <c r="H84" s="3" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
     </row>
     <row r="85" spans="1:8">
@@ -25873,7 +25873,7 @@
         <v>214</v>
       </c>
       <c r="H85" s="6" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
     </row>
     <row r="86" spans="1:8">
@@ -25925,7 +25925,7 @@
         <v>220</v>
       </c>
       <c r="H87" s="6" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
     </row>
     <row r="88" spans="1:8" ht="43.2">
@@ -25951,7 +25951,7 @@
         <v>222</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
     </row>
     <row r="89" spans="1:8" ht="43.2">
@@ -25974,10 +25974,10 @@
         <v>12</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="H89" s="3" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
     </row>
     <row r="90" spans="1:8" ht="72">
@@ -26003,7 +26003,7 @@
         <v>226</v>
       </c>
       <c r="H90" s="3" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
     </row>
     <row r="91" spans="1:8" ht="72">
@@ -26029,7 +26029,7 @@
         <v>228</v>
       </c>
       <c r="H91" s="3" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
     </row>
     <row r="92" spans="1:8">
@@ -26081,7 +26081,7 @@
         <v>233</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
     </row>
     <row r="94" spans="1:8">
@@ -26107,7 +26107,7 @@
         <v>235</v>
       </c>
       <c r="H94" s="6" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
     </row>
     <row r="95" spans="1:8">
@@ -26133,7 +26133,7 @@
         <v>237</v>
       </c>
       <c r="H95" s="6" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
     </row>
     <row r="96" spans="1:8" ht="201.6">
@@ -26159,7 +26159,7 @@
         <v>240</v>
       </c>
       <c r="H96" s="3" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
     </row>
     <row r="97" spans="1:8" ht="28.8">
@@ -26185,7 +26185,7 @@
         <v>243</v>
       </c>
       <c r="H97" s="6" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
     </row>
     <row r="98" spans="1:8" ht="129.6">
@@ -26211,7 +26211,7 @@
         <v>245</v>
       </c>
       <c r="H98" s="3" t="s">
-        <v>784</v>
+        <v>781</v>
       </c>
     </row>
     <row r="99" spans="1:8" ht="86.4">
@@ -26237,7 +26237,7 @@
         <v>248</v>
       </c>
       <c r="H99" s="3" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
     </row>
     <row r="100" spans="1:8" ht="302.39999999999998">
@@ -26263,7 +26263,7 @@
         <v>250</v>
       </c>
       <c r="H100" s="3" t="s">
-        <v>748</v>
+        <v>745</v>
       </c>
     </row>
     <row r="101" spans="1:8" ht="28.8">
@@ -26289,7 +26289,7 @@
         <v>253</v>
       </c>
       <c r="H101" s="3" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
     </row>
     <row r="102" spans="1:8" ht="86.4">
@@ -26315,7 +26315,7 @@
         <v>255</v>
       </c>
       <c r="H102" s="3" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
     </row>
     <row r="103" spans="1:8">
@@ -26367,7 +26367,7 @@
         <v>260</v>
       </c>
       <c r="H104" s="6" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
     </row>
     <row r="105" spans="1:8">
@@ -26419,7 +26419,7 @@
         <v>265</v>
       </c>
       <c r="H106" s="6" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
     </row>
     <row r="107" spans="1:8">
@@ -26497,7 +26497,7 @@
         <v>273</v>
       </c>
       <c r="H109" s="6" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
     </row>
     <row r="110" spans="1:8" ht="43.2">
@@ -26523,7 +26523,7 @@
         <v>276</v>
       </c>
       <c r="H110" s="3" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
     </row>
     <row r="111" spans="1:8" ht="86.4">
@@ -26546,10 +26546,10 @@
         <v>12</v>
       </c>
       <c r="G111" s="8" t="s">
-        <v>742</v>
+        <v>739</v>
       </c>
       <c r="H111" s="3" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
     </row>
     <row r="112" spans="1:8">
@@ -26575,7 +26575,7 @@
         <v>279</v>
       </c>
       <c r="H112" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
     </row>
     <row r="113" spans="1:8">
@@ -26601,7 +26601,7 @@
         <v>281</v>
       </c>
       <c r="H113" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
     </row>
     <row r="114" spans="1:8">
@@ -26627,7 +26627,7 @@
         <v>283</v>
       </c>
       <c r="H114" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
     </row>
     <row r="115" spans="1:8">
@@ -26653,7 +26653,7 @@
         <v>285</v>
       </c>
       <c r="H115" s="6" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
     </row>
     <row r="116" spans="1:8" ht="43.2">
@@ -26679,7 +26679,7 @@
         <v>287</v>
       </c>
       <c r="H116" s="6" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
     </row>
     <row r="117" spans="1:8" ht="28.8">
@@ -26757,7 +26757,7 @@
         <v>295</v>
       </c>
       <c r="H119" s="6" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
     </row>
     <row r="120" spans="1:8" ht="28.8">
@@ -26783,7 +26783,7 @@
         <v>298</v>
       </c>
       <c r="H120" s="3" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
     </row>
     <row r="121" spans="1:8">
@@ -26809,7 +26809,7 @@
         <v>300</v>
       </c>
       <c r="H121" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
     </row>
     <row r="122" spans="1:8" ht="86.4">
@@ -26835,7 +26835,7 @@
         <v>303</v>
       </c>
       <c r="H122" s="3" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
     </row>
     <row r="123" spans="1:8" ht="28.8">
@@ -26861,7 +26861,7 @@
         <v>305</v>
       </c>
       <c r="H123" s="6" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
     </row>
     <row r="124" spans="1:8" ht="28.8">
@@ -26887,7 +26887,7 @@
         <v>307</v>
       </c>
       <c r="H124" s="8" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
     </row>
     <row r="125" spans="1:8" ht="28.8">
@@ -26913,7 +26913,7 @@
         <v>309</v>
       </c>
       <c r="H125" s="8" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
     </row>
     <row r="126" spans="1:8" ht="28.8">
@@ -26939,7 +26939,7 @@
         <v>311</v>
       </c>
       <c r="H126" s="8" t="s">
-        <v>731</v>
+        <v>728</v>
       </c>
     </row>
     <row r="127" spans="1:8">
@@ -26965,7 +26965,7 @@
         <v>313</v>
       </c>
       <c r="H127" s="8" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
     </row>
     <row r="128" spans="1:8">
@@ -27017,7 +27017,7 @@
         <v>318</v>
       </c>
       <c r="H129" s="3" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
     </row>
     <row r="130" spans="1:8">
@@ -27043,7 +27043,7 @@
         <v>320</v>
       </c>
       <c r="H130" s="3" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
     </row>
     <row r="131" spans="1:8" ht="28.8">
@@ -27069,7 +27069,7 @@
         <v>323</v>
       </c>
       <c r="H131" s="6" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
     </row>
     <row r="132" spans="1:8" ht="403.2">
@@ -27095,7 +27095,7 @@
         <v>325</v>
       </c>
       <c r="H132" s="3" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
     </row>
     <row r="133" spans="1:8">
@@ -27121,7 +27121,7 @@
         <v>328</v>
       </c>
       <c r="H133" s="6" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
     </row>
     <row r="134" spans="1:8" ht="43.2">
@@ -27131,23 +27131,23 @@
       <c r="B134" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="C134" s="2">
+      <c r="C134" s="10">
         <v>1</v>
       </c>
-      <c r="D134" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="E134" s="2" t="s">
+      <c r="D134" s="10" t="s">
+        <v>796</v>
+      </c>
+      <c r="E134" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="F134" s="2" t="s">
+      <c r="F134" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="G134" s="3" t="s">
-        <v>330</v>
+      <c r="G134" s="11" t="s">
+        <v>797</v>
       </c>
       <c r="H134" s="6" t="s">
-        <v>667</v>
+        <v>795</v>
       </c>
     </row>
     <row r="135" spans="1:8" ht="100.8">
@@ -27161,7 +27161,7 @@
         <v>2</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>753</v>
+        <v>750</v>
       </c>
       <c r="E135" s="2" t="s">
         <v>11</v>
@@ -27170,24 +27170,24 @@
         <v>12</v>
       </c>
       <c r="G135" s="3" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H135" s="3" t="s">
-        <v>732</v>
+        <v>729</v>
       </c>
     </row>
     <row r="136" spans="1:8" ht="115.2">
       <c r="A136" s="2" t="s">
-        <v>763</v>
+        <v>760</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="C136" s="2">
         <v>0</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
       <c r="E136" s="2" t="s">
         <v>11</v>
@@ -27196,10 +27196,10 @@
         <v>12</v>
       </c>
       <c r="G136" s="3" t="s">
-        <v>775</v>
+        <v>772</v>
       </c>
       <c r="H136" s="3" t="s">
-        <v>776</v>
+        <v>773</v>
       </c>
     </row>
     <row r="137" spans="1:8" ht="409.6">
@@ -27213,7 +27213,7 @@
         <v>3</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="E137" s="2" t="s">
         <v>11</v>
@@ -27222,10 +27222,10 @@
         <v>12</v>
       </c>
       <c r="G137" s="3" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="H137" s="3" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
     </row>
     <row r="138" spans="1:8" ht="28.8">
@@ -27233,13 +27233,13 @@
         <v>8</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C138" s="2">
         <v>1</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="E138" s="2" t="s">
         <v>11</v>
@@ -27248,10 +27248,10 @@
         <v>12</v>
       </c>
       <c r="G138" s="3" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="H138" s="6" t="s">
-        <v>668</v>
+        <v>665</v>
       </c>
     </row>
     <row r="139" spans="1:8">
@@ -27259,13 +27259,13 @@
         <v>8</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C139" s="2">
         <v>0</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="E139" s="2" t="s">
         <v>11</v>
@@ -27274,10 +27274,10 @@
         <v>12</v>
       </c>
       <c r="G139" s="3" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="H139" s="6" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
     </row>
     <row r="140" spans="1:8" ht="57.6">
@@ -27285,13 +27285,13 @@
         <v>8</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C140" s="2">
         <v>1</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="E140" s="2" t="s">
         <v>11</v>
@@ -27300,10 +27300,10 @@
         <v>12</v>
       </c>
       <c r="G140" s="3" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="H140" s="6" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
     </row>
     <row r="141" spans="1:8">
@@ -27311,13 +27311,13 @@
         <v>8</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C141" s="2">
         <v>2</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="E141" s="2" t="s">
         <v>11</v>
@@ -27326,10 +27326,10 @@
         <v>12</v>
       </c>
       <c r="G141" s="3" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="H141" s="6" t="s">
-        <v>671</v>
+        <v>668</v>
       </c>
     </row>
     <row r="142" spans="1:8" ht="43.2">
@@ -27337,13 +27337,13 @@
         <v>8</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C142" s="2">
         <v>3</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="E142" s="2" t="s">
         <v>11</v>
@@ -27352,10 +27352,10 @@
         <v>12</v>
       </c>
       <c r="G142" s="3" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="H142" s="6" t="s">
-        <v>672</v>
+        <v>669</v>
       </c>
     </row>
     <row r="143" spans="1:8" ht="86.4">
@@ -27363,13 +27363,13 @@
         <v>8</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C143" s="2">
         <v>4</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="E143" s="2" t="s">
         <v>11</v>
@@ -27378,10 +27378,10 @@
         <v>12</v>
       </c>
       <c r="G143" s="3" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="H143" s="3" t="s">
-        <v>673</v>
+        <v>670</v>
       </c>
     </row>
     <row r="144" spans="1:8" ht="216">
@@ -27389,13 +27389,13 @@
         <v>8</v>
       </c>
       <c r="B144" s="2" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C144" s="2">
         <v>5</v>
       </c>
       <c r="D144" s="2" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="E144" s="2" t="s">
         <v>11</v>
@@ -27404,10 +27404,10 @@
         <v>12</v>
       </c>
       <c r="G144" s="3" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="H144" s="3" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
     </row>
     <row r="145" spans="1:8" ht="86.4">
@@ -27415,13 +27415,13 @@
         <v>8</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C145" s="2">
         <v>0</v>
       </c>
       <c r="D145" s="2" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="E145" s="2" t="s">
         <v>11</v>
@@ -27430,10 +27430,10 @@
         <v>12</v>
       </c>
       <c r="G145" s="3" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="H145" s="3" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="146" spans="1:8" ht="86.4">
@@ -27441,13 +27441,13 @@
         <v>8</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C146" s="2">
         <v>1</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="E146" s="2" t="s">
         <v>11</v>
@@ -27456,10 +27456,10 @@
         <v>12</v>
       </c>
       <c r="G146" s="3" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="H146" s="3" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
     </row>
     <row r="147" spans="1:8">
@@ -27467,13 +27467,13 @@
         <v>8</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C147" s="2">
         <v>2</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="E147" s="2" t="s">
         <v>11</v>
@@ -27482,10 +27482,10 @@
         <v>12</v>
       </c>
       <c r="G147" s="3" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="H147" s="6" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="148" spans="1:8" ht="86.4">
@@ -27493,13 +27493,13 @@
         <v>8</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C148" s="2">
         <v>0</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="E148" s="2" t="s">
         <v>11</v>
@@ -27508,10 +27508,10 @@
         <v>12</v>
       </c>
       <c r="G148" s="3" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="H148" s="3" t="s">
-        <v>675</v>
+        <v>672</v>
       </c>
     </row>
     <row r="149" spans="1:8" ht="28.8">
@@ -27519,13 +27519,13 @@
         <v>8</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C149" s="2">
         <v>0</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="E149" s="2" t="s">
         <v>11</v>
@@ -27534,10 +27534,10 @@
         <v>12</v>
       </c>
       <c r="G149" s="3" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="H149" s="3" t="s">
-        <v>676</v>
+        <v>673</v>
       </c>
     </row>
     <row r="150" spans="1:8">
@@ -27545,13 +27545,13 @@
         <v>8</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C150" s="2">
         <v>2</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="E150" s="2" t="s">
         <v>11</v>
@@ -27560,10 +27560,10 @@
         <v>12</v>
       </c>
       <c r="G150" s="3" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="H150" s="3" t="s">
-        <v>677</v>
+        <v>674</v>
       </c>
     </row>
     <row r="151" spans="1:8" ht="129.6">
@@ -27571,13 +27571,13 @@
         <v>8</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C151" s="2">
         <v>0</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="E151" s="2" t="s">
         <v>11</v>
@@ -27586,10 +27586,10 @@
         <v>12</v>
       </c>
       <c r="G151" s="3" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="H151" s="3" t="s">
-        <v>758</v>
+        <v>755</v>
       </c>
     </row>
     <row r="152" spans="1:8" ht="28.8">
@@ -27597,13 +27597,13 @@
         <v>8</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C152" s="2">
         <v>1</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="E152" s="2" t="s">
         <v>11</v>
@@ -27612,10 +27612,10 @@
         <v>12</v>
       </c>
       <c r="G152" s="3" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="H152" s="6" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="153" spans="1:8" ht="28.8">
@@ -27623,13 +27623,13 @@
         <v>8</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C153" s="2">
         <v>0</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="E153" s="2" t="s">
         <v>11</v>
@@ -27638,10 +27638,10 @@
         <v>12</v>
       </c>
       <c r="G153" s="3" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="H153" s="3" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="154" spans="1:8" ht="115.2">
@@ -27649,13 +27649,13 @@
         <v>8</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C154" s="2">
         <v>1</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="E154" s="2" t="s">
         <v>11</v>
@@ -27664,10 +27664,10 @@
         <v>12</v>
       </c>
       <c r="G154" s="3" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="H154" s="3" t="s">
-        <v>678</v>
+        <v>675</v>
       </c>
     </row>
     <row r="155" spans="1:8" ht="28.8">
@@ -27675,13 +27675,13 @@
         <v>8</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="C155" s="2">
         <v>0</v>
       </c>
       <c r="D155" s="2" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="E155" s="2" t="s">
         <v>11</v>
@@ -27690,10 +27690,10 @@
         <v>12</v>
       </c>
       <c r="G155" s="3" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="H155" s="6" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
     </row>
     <row r="156" spans="1:8" ht="409.6">
@@ -27701,13 +27701,13 @@
         <v>8</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="C156" s="2">
         <v>1</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="E156" s="2" t="s">
         <v>11</v>
@@ -27716,10 +27716,10 @@
         <v>12</v>
       </c>
       <c r="G156" s="3" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="H156" s="3" t="s">
-        <v>733</v>
+        <v>730</v>
       </c>
     </row>
     <row r="157" spans="1:8" ht="43.2">
@@ -27727,13 +27727,13 @@
         <v>8</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="C157" s="2">
         <v>0</v>
       </c>
       <c r="D157" s="2" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="E157" s="2" t="s">
         <v>11</v>
@@ -27742,10 +27742,10 @@
         <v>12</v>
       </c>
       <c r="G157" s="3" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="H157" s="6" t="s">
-        <v>680</v>
+        <v>677</v>
       </c>
     </row>
     <row r="158" spans="1:8" ht="86.4">
@@ -27753,13 +27753,13 @@
         <v>8</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="C158" s="2">
         <v>1</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="E158" s="2" t="s">
         <v>11</v>
@@ -27768,10 +27768,10 @@
         <v>12</v>
       </c>
       <c r="G158" s="3" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="H158" s="3" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="159" spans="1:8" ht="28.8">
@@ -27779,13 +27779,13 @@
         <v>8</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="C159" s="2">
         <v>0</v>
       </c>
       <c r="D159" s="2" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="E159" s="2" t="s">
         <v>11</v>
@@ -27794,10 +27794,10 @@
         <v>12</v>
       </c>
       <c r="G159" s="3" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="H159" s="6" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="160" spans="1:8" ht="144">
@@ -27805,13 +27805,13 @@
         <v>8</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="C160" s="2">
         <v>1</v>
       </c>
       <c r="D160" s="2" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="E160" s="2" t="s">
         <v>11</v>
@@ -27820,10 +27820,10 @@
         <v>12</v>
       </c>
       <c r="G160" s="3" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="H160" s="6" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
     </row>
     <row r="161" spans="1:8" ht="100.8">
@@ -27831,13 +27831,13 @@
         <v>8</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C161" s="2">
         <v>0</v>
       </c>
       <c r="D161" s="2" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="E161" s="2" t="s">
         <v>11</v>
@@ -27846,10 +27846,10 @@
         <v>12</v>
       </c>
       <c r="G161" s="3" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="H161" s="3" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
     </row>
     <row r="162" spans="1:8" ht="144">
@@ -27857,13 +27857,13 @@
         <v>8</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C162" s="2">
         <v>1</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="E162" s="2" t="s">
         <v>11</v>
@@ -27872,10 +27872,10 @@
         <v>12</v>
       </c>
       <c r="G162" s="3" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="H162" s="3" t="s">
-        <v>735</v>
+        <v>732</v>
       </c>
     </row>
     <row r="163" spans="1:8" ht="100.8">
@@ -27883,13 +27883,13 @@
         <v>8</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C163" s="2">
         <v>0</v>
       </c>
       <c r="D163" s="2" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="E163" s="2" t="s">
         <v>11</v>
@@ -27898,10 +27898,10 @@
         <v>12</v>
       </c>
       <c r="G163" s="3" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="H163" s="3" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
     </row>
     <row r="164" spans="1:8" ht="43.2">
@@ -27909,13 +27909,13 @@
         <v>8</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C164" s="2">
         <v>1</v>
       </c>
       <c r="D164" s="2" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="E164" s="2" t="s">
         <v>11</v>
@@ -27924,10 +27924,10 @@
         <v>12</v>
       </c>
       <c r="G164" s="3" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="H164" s="6" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
     </row>
     <row r="165" spans="1:8" ht="115.2">
@@ -27935,13 +27935,13 @@
         <v>8</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="C165" s="2">
         <v>0</v>
       </c>
       <c r="D165" s="2" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="E165" s="2" t="s">
         <v>11</v>
@@ -27950,10 +27950,10 @@
         <v>12</v>
       </c>
       <c r="G165" s="3" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="H165" s="3" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
     </row>
     <row r="166" spans="1:8" ht="86.4">
@@ -27961,13 +27961,13 @@
         <v>8</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="C166" s="2">
         <v>1</v>
       </c>
       <c r="D166" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="E166" s="2" t="s">
         <v>11</v>
@@ -27976,10 +27976,10 @@
         <v>12</v>
       </c>
       <c r="G166" s="3" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="H166" s="3" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="167" spans="1:8" ht="86.4">
@@ -27987,13 +27987,13 @@
         <v>8</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="C167" s="2">
         <v>0</v>
       </c>
       <c r="D167" s="2" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="E167" s="2" t="s">
         <v>11</v>
@@ -28002,10 +28002,10 @@
         <v>12</v>
       </c>
       <c r="G167" s="3" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="H167" s="3" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="168" spans="1:8" ht="28.8">
@@ -28013,13 +28013,13 @@
         <v>8</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="C168" s="2">
         <v>0</v>
       </c>
       <c r="D168" s="2" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="E168" s="2" t="s">
         <v>11</v>
@@ -28028,10 +28028,10 @@
         <v>12</v>
       </c>
       <c r="G168" s="3" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="H168" s="3" t="s">
-        <v>736</v>
+        <v>733</v>
       </c>
     </row>
     <row r="169" spans="1:8" ht="57.6">
@@ -28039,13 +28039,13 @@
         <v>8</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="C169" s="2">
         <v>1</v>
       </c>
       <c r="D169" s="2" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="E169" s="2" t="s">
         <v>11</v>
@@ -28054,10 +28054,10 @@
         <v>12</v>
       </c>
       <c r="G169" s="3" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="H169" s="3" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="170" spans="1:8">
@@ -28065,13 +28065,13 @@
         <v>8</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="C170" s="2">
         <v>2</v>
       </c>
       <c r="D170" s="2" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="E170" s="2" t="s">
         <v>11</v>
@@ -28080,10 +28080,10 @@
         <v>12</v>
       </c>
       <c r="G170" s="3" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="H170" s="3" t="s">
-        <v>694</v>
+        <v>691</v>
       </c>
     </row>
     <row r="171" spans="1:8" ht="57.6">
@@ -28091,13 +28091,13 @@
         <v>8</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="C171" s="2">
         <v>0</v>
       </c>
       <c r="D171" s="2" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="E171" s="2" t="s">
         <v>11</v>
@@ -28106,10 +28106,10 @@
         <v>12</v>
       </c>
       <c r="G171" s="3" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="H171" s="6" t="s">
-        <v>695</v>
+        <v>692</v>
       </c>
     </row>
     <row r="172" spans="1:8" ht="28.8">
@@ -28117,13 +28117,13 @@
         <v>8</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="C172" s="2">
         <v>1</v>
       </c>
       <c r="D172" s="2" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="E172" s="2" t="s">
         <v>11</v>
@@ -28132,10 +28132,10 @@
         <v>12</v>
       </c>
       <c r="G172" s="3" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="H172" s="6" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="173" spans="1:8" ht="28.8">
@@ -28143,13 +28143,13 @@
         <v>8</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="C173" s="2">
         <v>0</v>
       </c>
       <c r="D173" s="2" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="E173" s="2" t="s">
         <v>11</v>
@@ -28158,10 +28158,10 @@
         <v>12</v>
       </c>
       <c r="G173" s="3" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="H173" s="6" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="174" spans="1:8" ht="409.6">
@@ -28169,13 +28169,13 @@
         <v>8</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="C174" s="2">
         <v>1</v>
       </c>
       <c r="D174" s="2" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="E174" s="2" t="s">
         <v>11</v>
@@ -28184,10 +28184,10 @@
         <v>12</v>
       </c>
       <c r="G174" s="3" t="s">
-        <v>696</v>
+        <v>693</v>
       </c>
       <c r="H174" s="3" t="s">
-        <v>737</v>
+        <v>734</v>
       </c>
     </row>
     <row r="175" spans="1:8" ht="28.8">
@@ -28195,13 +28195,13 @@
         <v>8</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="C175" s="2">
         <v>0</v>
       </c>
       <c r="D175" s="2" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="E175" s="2" t="s">
         <v>11</v>
@@ -28210,10 +28210,10 @@
         <v>12</v>
       </c>
       <c r="G175" s="3" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="H175" s="6" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="176" spans="1:8" ht="409.6">
@@ -28221,13 +28221,13 @@
         <v>8</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="C176" s="2">
         <v>1</v>
       </c>
       <c r="D176" s="2" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
       <c r="E176" s="2" t="s">
         <v>11</v>
@@ -28236,10 +28236,10 @@
         <v>12</v>
       </c>
       <c r="G176" s="3" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
       <c r="H176" s="3" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
     </row>
     <row r="177" spans="1:8" ht="201.6">
@@ -28247,13 +28247,13 @@
         <v>8</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="C177" s="2">
         <v>2</v>
       </c>
       <c r="D177" s="2" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E177" s="2" t="s">
         <v>11</v>
@@ -28262,10 +28262,10 @@
         <v>12</v>
       </c>
       <c r="G177" s="3" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="H177" s="3" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
     </row>
     <row r="178" spans="1:8" ht="86.4">
@@ -28273,13 +28273,13 @@
         <v>8</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="C178" s="2">
         <v>0</v>
       </c>
       <c r="D178" s="2" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="E178" s="2" t="s">
         <v>11</v>
@@ -28288,10 +28288,10 @@
         <v>12</v>
       </c>
       <c r="G178" s="3" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="H178" s="3" t="s">
-        <v>759</v>
+        <v>756</v>
       </c>
     </row>
     <row r="179" spans="1:8">
@@ -28299,13 +28299,13 @@
         <v>8</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="C179" s="2">
         <v>1</v>
       </c>
       <c r="D179" s="2" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="E179" s="2" t="s">
         <v>11</v>
@@ -28314,7 +28314,7 @@
         <v>12</v>
       </c>
       <c r="G179" s="3" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="H179" s="6" t="s">
         <v>29</v>
@@ -28325,13 +28325,13 @@
         <v>8</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="C180" s="2">
         <v>0</v>
       </c>
       <c r="D180" s="2" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="E180" s="2" t="s">
         <v>11</v>
@@ -28340,10 +28340,10 @@
         <v>12</v>
       </c>
       <c r="G180" s="3" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="H180" s="6" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
     </row>
     <row r="181" spans="1:8">
@@ -28351,13 +28351,13 @@
         <v>8</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="C181" s="2">
         <v>0</v>
       </c>
       <c r="D181" s="2" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="E181" s="2" t="s">
         <v>11</v>
@@ -28366,10 +28366,10 @@
         <v>12</v>
       </c>
       <c r="G181" s="3" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="H181" s="6" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
     </row>
     <row r="182" spans="1:8">
@@ -28377,13 +28377,13 @@
         <v>8</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="C182" s="2">
         <v>0</v>
       </c>
       <c r="D182" s="2" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="E182" s="2" t="s">
         <v>11</v>
@@ -28392,10 +28392,10 @@
         <v>12</v>
       </c>
       <c r="G182" s="3" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="H182" s="6" t="s">
-        <v>698</v>
+        <v>695</v>
       </c>
     </row>
     <row r="183" spans="1:8">
@@ -28403,13 +28403,13 @@
         <v>8</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="C183" s="2">
         <v>0</v>
       </c>
       <c r="D183" s="2" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="E183" s="2" t="s">
         <v>11</v>
@@ -28418,10 +28418,10 @@
         <v>12</v>
       </c>
       <c r="G183" s="3" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="H183" s="6" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
     </row>
     <row r="184" spans="1:8">
@@ -28429,13 +28429,13 @@
         <v>8</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="C184" s="2">
         <v>0</v>
       </c>
       <c r="D184" s="2" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="E184" s="2" t="s">
         <v>11</v>
@@ -28444,10 +28444,10 @@
         <v>12</v>
       </c>
       <c r="G184" s="3" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="H184" s="6" t="s">
-        <v>699</v>
+        <v>696</v>
       </c>
     </row>
     <row r="185" spans="1:8" ht="144">
@@ -28455,13 +28455,13 @@
         <v>8</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C185" s="2">
         <v>0</v>
       </c>
       <c r="D185" s="2" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="E185" s="2" t="s">
         <v>11</v>
@@ -28470,10 +28470,10 @@
         <v>12</v>
       </c>
       <c r="G185" s="3" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="H185" s="3" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
     </row>
     <row r="186" spans="1:8" ht="28.8">
@@ -28481,13 +28481,13 @@
         <v>8</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C186" s="2">
         <v>14</v>
       </c>
       <c r="D186" s="2" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="E186" s="2" t="s">
         <v>11</v>
@@ -28496,10 +28496,10 @@
         <v>12</v>
       </c>
       <c r="G186" s="3" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="H186" s="6" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
     </row>
     <row r="187" spans="1:8" ht="28.8">
@@ -28507,13 +28507,13 @@
         <v>8</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C187" s="2">
         <v>15</v>
       </c>
       <c r="D187" s="2" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="E187" s="2" t="s">
         <v>11</v>
@@ -28522,10 +28522,10 @@
         <v>12</v>
       </c>
       <c r="G187" s="3" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="H187" s="6" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
     <row r="188" spans="1:8" ht="57.6">
@@ -28533,13 +28533,13 @@
         <v>8</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C188" s="2">
         <v>16</v>
       </c>
       <c r="D188" s="2" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="E188" s="2" t="s">
         <v>11</v>
@@ -28548,10 +28548,10 @@
         <v>12</v>
       </c>
       <c r="G188" s="3" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="H188" s="3" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
     <row r="189" spans="1:8" ht="28.8">
@@ -28559,13 +28559,13 @@
         <v>8</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C189" s="2">
         <v>18</v>
       </c>
       <c r="D189" s="2" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="E189" s="2" t="s">
         <v>11</v>
@@ -28574,10 +28574,10 @@
         <v>12</v>
       </c>
       <c r="G189" s="3" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="H189" s="6" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="190" spans="1:8" ht="57.6">
@@ -28585,13 +28585,13 @@
         <v>8</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C190" s="2">
         <v>20</v>
       </c>
       <c r="D190" s="2" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="E190" s="2" t="s">
         <v>11</v>
@@ -28600,10 +28600,10 @@
         <v>12</v>
       </c>
       <c r="G190" s="3" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="H190" s="3" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
     </row>
     <row r="191" spans="1:8" ht="43.2">
@@ -28611,13 +28611,13 @@
         <v>8</v>
       </c>
       <c r="B191" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C191" s="2">
         <v>21</v>
       </c>
       <c r="D191" s="2" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="E191" s="2" t="s">
         <v>11</v>
@@ -28626,10 +28626,10 @@
         <v>12</v>
       </c>
       <c r="G191" s="3" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="H191" s="6" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
     </row>
     <row r="192" spans="1:8" ht="28.8">
@@ -28637,13 +28637,13 @@
         <v>8</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C192" s="2">
         <v>22</v>
       </c>
       <c r="D192" s="2" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="E192" s="2" t="s">
         <v>11</v>
@@ -28652,10 +28652,10 @@
         <v>12</v>
       </c>
       <c r="G192" s="3" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="H192" s="6" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
     </row>
     <row r="193" spans="1:8" ht="28.8">
@@ -28663,13 +28663,13 @@
         <v>8</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C193" s="2">
         <v>29</v>
       </c>
       <c r="D193" s="2" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="E193" s="2" t="s">
         <v>11</v>
@@ -28678,10 +28678,10 @@
         <v>12</v>
       </c>
       <c r="G193" s="3" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="H193" s="6" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="194" spans="1:8" ht="244.8">
@@ -28689,13 +28689,13 @@
         <v>8</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C194" s="2">
         <v>30</v>
       </c>
       <c r="D194" s="2" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="E194" s="2" t="s">
         <v>11</v>
@@ -28704,10 +28704,10 @@
         <v>12</v>
       </c>
       <c r="G194" s="3" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="H194" s="6" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
     </row>
     <row r="195" spans="1:8">
@@ -28715,13 +28715,13 @@
         <v>8</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C195" s="2">
         <v>31</v>
       </c>
       <c r="D195" s="2" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="E195" s="2" t="s">
         <v>11</v>
@@ -28730,7 +28730,7 @@
         <v>12</v>
       </c>
       <c r="G195" s="3" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="H195" s="6" t="s">
         <v>14</v>
@@ -28741,13 +28741,13 @@
         <v>8</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C196" s="2">
         <v>0</v>
       </c>
       <c r="D196" s="2" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="E196" s="2" t="s">
         <v>11</v>
@@ -28756,10 +28756,10 @@
         <v>12</v>
       </c>
       <c r="G196" s="3" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="H196" s="6" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
     </row>
     <row r="197" spans="1:8" ht="28.8">
@@ -28767,13 +28767,13 @@
         <v>8</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C197" s="2">
         <v>1</v>
       </c>
       <c r="D197" s="2" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="E197" s="2" t="s">
         <v>11</v>
@@ -28782,10 +28782,10 @@
         <v>12</v>
       </c>
       <c r="G197" s="3" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="H197" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
     </row>
     <row r="198" spans="1:8">
@@ -28793,13 +28793,13 @@
         <v>8</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C198" s="2">
         <v>2</v>
       </c>
       <c r="D198" s="2" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="E198" s="2" t="s">
         <v>11</v>
@@ -28808,10 +28808,10 @@
         <v>12</v>
       </c>
       <c r="G198" s="3" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="H198" s="6" t="s">
-        <v>739</v>
+        <v>736</v>
       </c>
     </row>
     <row r="199" spans="1:8" ht="100.8">
@@ -28819,13 +28819,13 @@
         <v>8</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C199" s="2">
         <v>3</v>
       </c>
       <c r="D199" s="2" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="E199" s="2" t="s">
         <v>11</v>
@@ -28834,10 +28834,10 @@
         <v>12</v>
       </c>
       <c r="G199" s="3" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="H199" s="3" t="s">
-        <v>760</v>
+        <v>757</v>
       </c>
     </row>
     <row r="200" spans="1:8" ht="158.4">
@@ -28845,13 +28845,13 @@
         <v>8</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C200" s="2">
         <v>4</v>
       </c>
       <c r="D200" s="2" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="E200" s="2" t="s">
         <v>11</v>
@@ -28860,10 +28860,10 @@
         <v>12</v>
       </c>
       <c r="G200" s="3" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="H200" s="3" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
     </row>
     <row r="201" spans="1:8" ht="43.2">
@@ -28871,13 +28871,13 @@
         <v>8</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C201" s="2">
         <v>5</v>
       </c>
       <c r="D201" s="2" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="E201" s="2" t="s">
         <v>11</v>
@@ -28886,10 +28886,10 @@
         <v>12</v>
       </c>
       <c r="G201" s="3" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="H201" s="3" t="s">
-        <v>705</v>
+        <v>702</v>
       </c>
     </row>
     <row r="202" spans="1:8" ht="100.8">
@@ -28897,13 +28897,13 @@
         <v>8</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C202" s="2">
         <v>6</v>
       </c>
       <c r="D202" s="2" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="E202" s="2" t="s">
         <v>11</v>
@@ -28912,10 +28912,10 @@
         <v>12</v>
       </c>
       <c r="G202" s="3" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="H202" s="3" t="s">
-        <v>706</v>
+        <v>703</v>
       </c>
     </row>
     <row r="203" spans="1:8" ht="43.2">
@@ -28923,13 +28923,13 @@
         <v>8</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C203" s="2">
         <v>7</v>
       </c>
       <c r="D203" s="2" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="E203" s="2" t="s">
         <v>11</v>
@@ -28938,10 +28938,10 @@
         <v>12</v>
       </c>
       <c r="G203" s="3" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="H203" s="3" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
     </row>
     <row r="204" spans="1:8" ht="100.8">
@@ -28949,13 +28949,13 @@
         <v>8</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C204" s="2">
         <v>8</v>
       </c>
       <c r="D204" s="2" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="E204" s="2" t="s">
         <v>11</v>
@@ -28964,10 +28964,10 @@
         <v>12</v>
       </c>
       <c r="G204" s="3" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="H204" s="3" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
     </row>
     <row r="205" spans="1:8" ht="100.8">
@@ -28975,13 +28975,13 @@
         <v>8</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C205" s="2">
         <v>9</v>
       </c>
       <c r="D205" s="2" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="E205" s="2" t="s">
         <v>11</v>
@@ -28990,10 +28990,10 @@
         <v>12</v>
       </c>
       <c r="G205" s="3" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="H205" s="3" t="s">
-        <v>740</v>
+        <v>737</v>
       </c>
     </row>
     <row r="206" spans="1:8" ht="115.2">
@@ -29001,13 +29001,13 @@
         <v>8</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C206" s="2">
         <v>10</v>
       </c>
       <c r="D206" s="2" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="E206" s="2" t="s">
         <v>11</v>
@@ -29016,10 +29016,10 @@
         <v>12</v>
       </c>
       <c r="G206" s="3" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="H206" s="3" t="s">
-        <v>709</v>
+        <v>706</v>
       </c>
     </row>
     <row r="207" spans="1:8" ht="158.4">
@@ -29027,13 +29027,13 @@
         <v>8</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C207" s="2">
         <v>11</v>
       </c>
       <c r="D207" s="2" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="E207" s="2" t="s">
         <v>11</v>
@@ -29042,10 +29042,10 @@
         <v>12</v>
       </c>
       <c r="G207" s="3" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="H207" s="3" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
     </row>
     <row r="208" spans="1:8" ht="172.8">
@@ -29053,13 +29053,13 @@
         <v>8</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C208" s="2">
         <v>12</v>
       </c>
       <c r="D208" s="2" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="E208" s="2" t="s">
         <v>11</v>
@@ -29068,10 +29068,10 @@
         <v>12</v>
       </c>
       <c r="G208" s="3" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="H208" s="3" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
     </row>
     <row r="209" spans="1:9" ht="115.2">
@@ -29079,13 +29079,13 @@
         <v>8</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C209" s="2">
         <v>13</v>
       </c>
       <c r="D209" s="2" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="E209" s="2" t="s">
         <v>11</v>
@@ -29094,10 +29094,10 @@
         <v>12</v>
       </c>
       <c r="G209" s="3" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="H209" s="3" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
     </row>
     <row r="210" spans="1:9" ht="158.4">
@@ -29105,13 +29105,13 @@
         <v>8</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C210" s="2">
         <v>14</v>
       </c>
       <c r="D210" s="2" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="E210" s="2" t="s">
         <v>11</v>
@@ -29120,10 +29120,10 @@
         <v>12</v>
       </c>
       <c r="G210" s="3" t="s">
-        <v>761</v>
+        <v>758</v>
       </c>
       <c r="H210" s="3" t="s">
-        <v>762</v>
+        <v>759</v>
       </c>
     </row>
     <row r="211" spans="1:9" ht="158.4">
@@ -29131,13 +29131,13 @@
         <v>8</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C211" s="2">
         <v>15</v>
       </c>
       <c r="D211" s="2" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="E211" s="2" t="s">
         <v>11</v>
@@ -29146,10 +29146,10 @@
         <v>12</v>
       </c>
       <c r="G211" s="3" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="H211" s="3" t="s">
-        <v>713</v>
+        <v>710</v>
       </c>
     </row>
     <row r="212" spans="1:9" ht="100.8">
@@ -29157,13 +29157,13 @@
         <v>8</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C212" s="2">
         <v>16</v>
       </c>
       <c r="D212" s="2" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="E212" s="2" t="s">
         <v>11</v>
@@ -29172,10 +29172,10 @@
         <v>12</v>
       </c>
       <c r="G212" s="3" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="H212" s="3" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
     </row>
     <row r="213" spans="1:9" ht="100.8">
@@ -29183,13 +29183,13 @@
         <v>8</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C213" s="2">
         <v>17</v>
       </c>
       <c r="D213" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="E213" s="2" t="s">
         <v>11</v>
@@ -29198,10 +29198,10 @@
         <v>12</v>
       </c>
       <c r="G213" s="3" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="H213" s="3" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
     </row>
     <row r="214" spans="1:9" ht="43.2">
@@ -29209,13 +29209,13 @@
         <v>8</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C214" s="2">
         <v>18</v>
       </c>
       <c r="D214" s="2" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="E214" s="2" t="s">
         <v>11</v>
@@ -29224,10 +29224,10 @@
         <v>12</v>
       </c>
       <c r="G214" s="3" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="H214" s="3" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
     </row>
     <row r="215" spans="1:9" ht="43.2">
@@ -29235,13 +29235,13 @@
         <v>8</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C215" s="2">
         <v>19</v>
       </c>
       <c r="D215" s="2" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="E215" s="2" t="s">
         <v>11</v>
@@ -29250,10 +29250,10 @@
         <v>12</v>
       </c>
       <c r="G215" s="3" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="H215" s="3" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
     </row>
     <row r="216" spans="1:9" ht="43.2">
@@ -29261,13 +29261,13 @@
         <v>8</v>
       </c>
       <c r="B216" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C216" s="2">
         <v>20</v>
       </c>
       <c r="D216" s="2" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="E216" s="2" t="s">
         <v>11</v>
@@ -29276,10 +29276,10 @@
         <v>12</v>
       </c>
       <c r="G216" s="3" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="H216" s="3" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
     </row>
     <row r="217" spans="1:9" ht="409.6">
@@ -29287,13 +29287,13 @@
         <v>8</v>
       </c>
       <c r="B217" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C217" s="2">
         <v>21</v>
       </c>
       <c r="D217" s="2" t="s">
-        <v>787</v>
+        <v>784</v>
       </c>
       <c r="E217" s="2" t="s">
         <v>11</v>
@@ -29302,10 +29302,10 @@
         <v>12</v>
       </c>
       <c r="G217" s="3" t="s">
-        <v>788</v>
+        <v>785</v>
       </c>
       <c r="H217" s="3" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="I217" s="3"/>
     </row>
@@ -29314,13 +29314,13 @@
         <v>8</v>
       </c>
       <c r="B218" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C218" s="2">
         <v>22</v>
       </c>
       <c r="D218" s="2" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="E218" s="2" t="s">
         <v>11</v>
@@ -29329,10 +29329,10 @@
         <v>12</v>
       </c>
       <c r="G218" s="3" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="H218" s="3" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
     </row>
     <row r="219" spans="1:9" ht="43.2">
@@ -29340,13 +29340,13 @@
         <v>8</v>
       </c>
       <c r="B219" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C219" s="2">
         <v>23</v>
       </c>
       <c r="D219" s="2" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="E219" s="2" t="s">
         <v>11</v>
@@ -29355,10 +29355,10 @@
         <v>12</v>
       </c>
       <c r="G219" s="3" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="H219" s="3" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
     </row>
     <row r="220" spans="1:9" ht="86.4">
@@ -29366,13 +29366,13 @@
         <v>8</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C220" s="2">
         <v>24</v>
       </c>
       <c r="D220" s="2" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="E220" s="2" t="s">
         <v>11</v>
@@ -29381,10 +29381,10 @@
         <v>12</v>
       </c>
       <c r="G220" s="3" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="H220" s="3" t="s">
-        <v>685</v>
+        <v>682</v>
       </c>
     </row>
     <row r="221" spans="1:9" ht="115.2">
@@ -29392,13 +29392,13 @@
         <v>8</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C221" s="2">
         <v>25</v>
       </c>
       <c r="D221" s="2" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="E221" s="2" t="s">
         <v>11</v>
@@ -29407,10 +29407,10 @@
         <v>12</v>
       </c>
       <c r="G221" s="3" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="H221" s="3" t="s">
-        <v>686</v>
+        <v>683</v>
       </c>
     </row>
     <row r="222" spans="1:9" ht="43.2">
@@ -29418,13 +29418,13 @@
         <v>8</v>
       </c>
       <c r="B222" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C222" s="2">
         <v>26</v>
       </c>
       <c r="D222" s="2" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="E222" s="2" t="s">
         <v>11</v>
@@ -29433,10 +29433,10 @@
         <v>12</v>
       </c>
       <c r="G222" s="3" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="H222" s="3" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
     </row>
     <row r="223" spans="1:9" ht="100.8">
@@ -29444,13 +29444,13 @@
         <v>8</v>
       </c>
       <c r="B223" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C223" s="2">
         <v>27</v>
       </c>
       <c r="D223" s="2" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="E223" s="2" t="s">
         <v>11</v>
@@ -29459,10 +29459,10 @@
         <v>12</v>
       </c>
       <c r="G223" s="3" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="H223" s="3" t="s">
-        <v>741</v>
+        <v>738</v>
       </c>
     </row>
     <row r="224" spans="1:9" ht="43.2">
@@ -29470,13 +29470,13 @@
         <v>8</v>
       </c>
       <c r="B224" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C224" s="2">
         <v>28</v>
       </c>
       <c r="D224" s="2" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="E224" s="2" t="s">
         <v>11</v>
@@ -29485,10 +29485,10 @@
         <v>12</v>
       </c>
       <c r="G224" s="3" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="H224" s="3" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
     </row>
     <row r="225" spans="1:8" ht="43.2">
@@ -29496,13 +29496,13 @@
         <v>8</v>
       </c>
       <c r="B225" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C225" s="2">
         <v>29</v>
       </c>
       <c r="D225" s="2" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="E225" s="2" t="s">
         <v>11</v>
@@ -29511,10 +29511,10 @@
         <v>12</v>
       </c>
       <c r="G225" s="3" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="H225" s="3" t="s">
-        <v>688</v>
+        <v>685</v>
       </c>
     </row>
     <row r="226" spans="1:8" ht="100.8">
@@ -29522,13 +29522,13 @@
         <v>8</v>
       </c>
       <c r="B226" s="2" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C226" s="2">
         <v>30</v>
       </c>
       <c r="D226" s="2" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="E226" s="2" t="s">
         <v>11</v>
@@ -29537,10 +29537,10 @@
         <v>12</v>
       </c>
       <c r="G226" s="3" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="H226" s="3" t="s">
-        <v>689</v>
+        <v>686</v>
       </c>
     </row>
     <row r="227" spans="1:8" ht="28.8">
@@ -29548,13 +29548,13 @@
         <v>8</v>
       </c>
       <c r="B227" s="2" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="C227" s="2">
         <v>0</v>
       </c>
       <c r="D227" s="2" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="E227" s="2" t="s">
         <v>11</v>
@@ -29563,10 +29563,10 @@
         <v>12</v>
       </c>
       <c r="G227" s="3" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="H227" s="6" t="s">
-        <v>690</v>
+        <v>687</v>
       </c>
     </row>
     <row r="228" spans="1:8" ht="28.8">
@@ -29574,13 +29574,13 @@
         <v>8</v>
       </c>
       <c r="B228" s="2" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="C228" s="2">
         <v>0</v>
       </c>
       <c r="D228" s="2" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="E228" s="2" t="s">
         <v>11</v>
@@ -29589,10 +29589,10 @@
         <v>12</v>
       </c>
       <c r="G228" s="3" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="H228" s="3" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
     </row>
     <row r="229" spans="1:8" ht="43.2">
@@ -29600,13 +29600,13 @@
         <v>8</v>
       </c>
       <c r="B229" s="2" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="C229" s="2">
         <v>1</v>
       </c>
       <c r="D229" s="2" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="E229" s="2" t="s">
         <v>11</v>
@@ -29615,10 +29615,10 @@
         <v>12</v>
       </c>
       <c r="G229" s="3" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="H229" s="3" t="s">
-        <v>691</v>
+        <v>688</v>
       </c>
     </row>
     <row r="230" spans="1:8" ht="100.8">
@@ -29626,13 +29626,13 @@
         <v>8</v>
       </c>
       <c r="B230" s="2" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="C230" s="2">
         <v>2</v>
       </c>
       <c r="D230" s="2" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="E230" s="2" t="s">
         <v>11</v>
@@ -29641,10 +29641,10 @@
         <v>12</v>
       </c>
       <c r="G230" s="3" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="H230" s="3" t="s">
-        <v>692</v>
+        <v>689</v>
       </c>
     </row>
     <row r="231" spans="1:8" ht="43.2">
@@ -29652,13 +29652,13 @@
         <v>8</v>
       </c>
       <c r="B231" s="2" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="C231" s="2">
         <v>3</v>
       </c>
       <c r="D231" s="2" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="E231" s="2" t="s">
         <v>11</v>
@@ -29667,10 +29667,10 @@
         <v>12</v>
       </c>
       <c r="G231" s="3" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="H231" s="3" t="s">
-        <v>693</v>
+        <v>690</v>
       </c>
     </row>
     <row r="232" spans="1:8">
@@ -29678,13 +29678,13 @@
         <v>8</v>
       </c>
       <c r="B232" s="2" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="C232" s="2">
         <v>0</v>
       </c>
       <c r="D232" s="2" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="E232" s="2" t="s">
         <v>11</v>
@@ -29693,10 +29693,10 @@
         <v>12</v>
       </c>
       <c r="G232" s="3" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="H232" s="6" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
     </row>
     <row r="233" spans="1:8">
@@ -29704,13 +29704,13 @@
         <v>8</v>
       </c>
       <c r="B233" s="2" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="C233" s="2">
         <v>0</v>
       </c>
       <c r="D233" s="2" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="E233" s="2" t="s">
         <v>11</v>
@@ -29719,10 +29719,10 @@
         <v>12</v>
       </c>
       <c r="G233" s="3" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="H233" s="6" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
     </row>
     <row r="234" spans="1:8" ht="28.8">
@@ -29730,13 +29730,13 @@
         <v>8</v>
       </c>
       <c r="B234" s="2" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="C234" s="2">
         <v>1</v>
       </c>
       <c r="D234" s="2" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="E234" s="2" t="s">
         <v>11</v>
@@ -29745,10 +29745,10 @@
         <v>12</v>
       </c>
       <c r="G234" s="3" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="H234" s="6" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
     </row>
     <row r="235" spans="1:8">
@@ -29756,13 +29756,13 @@
         <v>8</v>
       </c>
       <c r="B235" s="2" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="C235" s="2">
         <v>0</v>
       </c>
       <c r="D235" s="2" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="E235" s="2" t="s">
         <v>11</v>
@@ -29771,10 +29771,10 @@
         <v>12</v>
       </c>
       <c r="G235" s="3" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="H235" s="6" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
     </row>
     <row r="236" spans="1:8" ht="28.8">
@@ -29782,13 +29782,13 @@
         <v>8</v>
       </c>
       <c r="B236" s="2" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="C236" s="2">
         <v>1</v>
       </c>
       <c r="D236" s="2" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="E236" s="2" t="s">
         <v>11</v>
@@ -29797,10 +29797,10 @@
         <v>12</v>
       </c>
       <c r="G236" s="3" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="H236" s="4" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
     </row>
     <row r="237" spans="1:8">
@@ -29808,13 +29808,13 @@
         <v>8</v>
       </c>
       <c r="B237" s="2" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="C237" s="2">
         <v>0</v>
       </c>
       <c r="D237" s="2" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="E237" s="2" t="s">
         <v>11</v>
@@ -29823,7 +29823,7 @@
         <v>12</v>
       </c>
       <c r="G237" s="3" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="H237" s="4" t="s">
         <v>23</v>
@@ -29834,13 +29834,13 @@
         <v>8</v>
       </c>
       <c r="B238" s="2" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="C238" s="2">
         <v>1</v>
       </c>
       <c r="D238" s="2" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="E238" s="2" t="s">
         <v>11</v>
@@ -29849,10 +29849,10 @@
         <v>12</v>
       </c>
       <c r="G238" s="3" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="H238" s="4" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
     </row>
     <row r="239" spans="1:8">
@@ -29860,13 +29860,13 @@
         <v>8</v>
       </c>
       <c r="B239" s="2" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="C239" s="2">
         <v>0</v>
       </c>
       <c r="D239" s="2" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="E239" s="2" t="s">
         <v>11</v>
@@ -29875,24 +29875,24 @@
         <v>12</v>
       </c>
       <c r="G239" s="3" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="H239" s="4" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
     </row>
     <row r="240" spans="1:8">
       <c r="A240" t="s">
-        <v>763</v>
+        <v>760</v>
       </c>
       <c r="B240" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="C240">
         <v>1</v>
       </c>
       <c r="D240" t="s">
-        <v>764</v>
+        <v>761</v>
       </c>
       <c r="E240" t="s">
         <v>11</v>
@@ -29901,10 +29901,10 @@
         <v>12</v>
       </c>
       <c r="G240" t="s">
-        <v>765</v>
+        <v>762</v>
       </c>
       <c r="H240" s="4" t="s">
-        <v>766</v>
+        <v>763</v>
       </c>
     </row>
     <row r="241" spans="1:8">

</xml_diff>